<commit_message>
updated task 6 after updating qwen to run after 6.1.6
</commit_message>
<xml_diff>
--- a/submissions/task_06_full_run.xlsx
+++ b/submissions/task_06_full_run.xlsx
@@ -575,27 +575,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>bad</t>
-        </is>
-      </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>bad</t>
+          <t>good</t>
         </is>
       </c>
       <c r="N2" t="inlineStr"/>
@@ -607,37 +607,37 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>The description starts with a clear and concise statement. The sentence structure is varied, with a mix of short and long sentences. However, the transition between the second and third sentences feels a bit abrupt, and the use of 'This' in the second sentence is a repeated sentence opener.</t>
+          <t>The description uses varied sentence structures and transitions smoothly between ideas. No two sentences start with the same word, and the flow feels natural and engaging. There is no robotic repetition or awkward phrasing.</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>There are no spelling, punctuation, or grammatical errors in the description. The sentence structure is clear and easy to follow.</t>
+          <t>There are no spelling, punctuation, or grammatical errors. All sentences are correctly structured and punctuated.</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>The description uses a sales-oriented tone, but it relies on only one persuasive technique, which is the emphasis on the features and benefits of the product. It does not use any emotional or aspirational language, and it does not create a sense of urgency.</t>
+          <t>The tone is persuasive and aspirational, using phrases like 'Experience the power and precision,' 'blazing-fast,' 'stunning,' and 'embrace the future of mobile technology.' These evoke emotional appeal and benefit framing, aligning with strong persuasive techniques.</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>The product description has 59 words, counted one by one.</t>
+          <t>The product description has 65 words, counted one by one.</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>The description mentions the product name (Apple iPhone 15 Pro), material (titanium frame and Ceramic Shield glass), and warranty (1-year limited warranty). However, it omits the attribute 'features' and the specific details about the display (120Hz ProMotion display) and charging (USB-C fast charging).</t>
+          <t>The description accurately mentions: Product Name (Apple iPhone 15 Pro), Material (titanium frame, Ceramic Shield glass), Warranty (1-year limited warranty), and all structured attributes (A17 Pro chip, 120 Hz ProMotion display, USB-C fast charging, compact). No hallucinated or invented details are present. All information is correctly and naturally integrated.</t>
         </is>
       </c>
       <c r="V2" t="n">
-        <v>11971.1</v>
+        <v>23201.8</v>
       </c>
       <c r="W2" t="n">
-        <v>1051</v>
+        <v>838</v>
       </c>
       <c r="X2" t="n">
-        <v>595</v>
+        <v>645</v>
       </c>
     </row>
     <row r="3">
@@ -677,7 +677,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -692,12 +692,12 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>good</t>
+          <t>bad</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>bad</t>
+          <t>good</t>
         </is>
       </c>
       <c r="N3" t="inlineStr"/>
@@ -709,37 +709,37 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>The description uses a mix of short and long sentences, but some of them are quite similar in structure. For example, 'Capture breathtaking moments...' and 'Delivers an incredibly smooth...' both start with a verb and have a similar rhythm. Additionally, the transition between sentences could be smoother, especially after 'while'.</t>
+          <t>The description uses varied sentence structures and transitions smoothly between ideas. No two sentences start with the same word, and the flow feels natural and engaging. There is no robotic repetition or awkward phrasing.</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>There are no spelling, punctuation, or grammatical errors in the description. The sentence structure is mostly correct, and the language is clear and concise.</t>
+          <t>There are no spelling, punctuation, or grammatical errors. All sentences are correctly structured and punctuated.</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>The description uses a persuasive tone, highlighting the phone's features and benefits. It appeals to the reader's desire for a high-quality smartphone and emphasizes the phone's durability and eco-friendliness. However, the language is not overly aggressive or emotional, and the tone is generally professional.</t>
+          <t>The tone is actively persuasive, using benefit framing (e.g., 'capture breathtaking moments', 'unleash your creativity'), aspirational language ('pinnacle of mobile technology', 'ultimate smartphone'), and emotional appeal ('built to last', 'eco-conscious choice'). These techniques collectively create a compelling, desire-driven narrative.</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>The product description has ?? words, counted one by one.</t>
+          <t>The product description has 98 words, counted one by one.</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>The description mentions the product name (Samsung Galaxy S24 Ultra), material (Armor Aluminum frame and Gorilla Glass Victus), and warranty (1-year limited warranty). However, it does not mention the 200MP camera or S-Pen support as attributes. The description also adds some minor details, such as 'cutting-edge imaging technology' and 'eco-conscious choice', which are not explicitly stated in the source data.</t>
+          <t>The description correctly includes the product name (Samsung Galaxy S24 Ultra), material (Armor Aluminum frame, Gorilla Glass Victus), and warranty (1-year limited warranty). All attributes (200MP camera, S-Pen support, 120Hz AMOLED, sustainably sourced) are accurately mentioned. No hallucinated or invented details are present. All information is grounded in the source data.</t>
         </is>
       </c>
       <c r="V3" t="n">
-        <v>14418.5</v>
+        <v>11919.7</v>
       </c>
       <c r="W3" t="n">
-        <v>1095</v>
+        <v>885</v>
       </c>
       <c r="X3" t="n">
-        <v>822</v>
+        <v>849</v>
       </c>
     </row>
     <row r="4">
@@ -779,27 +779,27 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>bad</t>
-        </is>
-      </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>bad</t>
+          <t>good</t>
         </is>
       </c>
       <c r="N4" t="inlineStr"/>
@@ -811,37 +811,37 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>The description flows well, but the first sentence starts with 'Capture', and the third sentence starts with 'The'. Additionally, the transition between the second and third sentences is a bit abrupt. However, the sentence structure is varied, and there are no robotic repetitions.</t>
+          <t>The description uses varied sentence structures and transitions smoothly between ideas. No two sentences start with the same word, and the flow feels natural and engaging. There is no robotic repetition or awkward phrasing.</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>There are no spelling, punctuation, or grammatical errors in the description. The sentence structure is clear, and the language is concise.</t>
+          <t>There are no spelling, punctuation, or grammatical errors. The sentence construction is correct and clear throughout.</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>The description uses a sales-oriented tone, but it relies on only one persuasive technique, which is the benefit framing of the Tensor G3 chip and Magic Eraser features. There is no emotional or aspirational appeal, and the language is not particularly engaging.</t>
+          <t>The tone is persuasive and aspirational, using benefit framing ('Capture life's magic', 'elevate your mobile experience') and sensory language ('breathtaking photos', 'premium style'). It also implies social proof through the high rating (implied by 'revolutionary' and 'stunning'), though not explicitly stated. Two distinct persuasive techniques are used.</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>The product description has 65 words, counted one by one.</t>
+          <t>The product description has 67 words, counted one by one.</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>The description mentions the Product Name (Google Pixel 8 Pro), Material (matte glass back and aluminum frame), and Warranty (1-year limited warranty). However, it omits the Attributes (Tensor G3 chip, Magic Eraser, 50MP camera) and Rating (4.7/5).</t>
+          <t>The description correctly mentions the Product Name (Google Pixel 8 Pro), Material (matte glass back, aluminum frame), and Warranty (1-year limited warranty). All structured attributes are included: Tensor G3 chip, Magic Eraser, 50MP camera. No hallucinated or invented details. All information is accurately represented and naturally integrated.</t>
         </is>
       </c>
       <c r="V4" t="n">
-        <v>9313.700000000001</v>
+        <v>38871.4</v>
       </c>
       <c r="W4" t="n">
-        <v>1052</v>
+        <v>832</v>
       </c>
       <c r="X4" t="n">
-        <v>607</v>
+        <v>666</v>
       </c>
     </row>
     <row r="5">
@@ -881,22 +881,22 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
           <t>ok</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>bad</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -913,37 +913,37 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>The description uses a mix of short and long sentences, but the transition between the second and third sentences feels a bit abrupt. Additionally, the sentence structure is mostly varied, but the last sentence starts with 'Backed', which is the same word that started the second sentence. However, the overall flow is still relatively smooth.</t>
+          <t>The description flows smoothly with varied sentence structure and natural transitions. No two sentences start with the same word. The phrasing is engaging and avoids robotic repetition. The rhythm feels conversational and polished.</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>The description appears to be free of any spelling, punctuation, or grammatical errors.</t>
+          <t>No spelling, punctuation, or grammatical errors are present. All sentences are properly structured and punctuated. The use of em dashes and commas is correct and enhances readability.</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>The description uses a persuasive tone by emphasizing the benefits of the product, such as 'fully immerse yourself in your music' and 'superior audio quality with confidence'. It also uses sensory language, like 'silencing distractions' and 'plush synthetic leather earcups', to create an aspirational appeal. However, it relies on only one persuasive technique, which is benefit framing.</t>
+          <t>The tone is persuasive and aspirational. It uses benefit framing ('escape into your own world of sound', 'fully immerse yourself'), emotional appeal ('perfect for long listening sessions'), and confidence-building language ('experience superior audio quality with confidence'). These techniques actively engage the reader beyond mere feature listing.</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>The product description has ?? words, counted one by one.</t>
+          <t>The product description has 86 words, counted one by one.</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>The description mentions the product name, material, and warranty, but it omits the attribute 'features' and 'capacity'. However, it does mention the battery life, which is a part of the 'features' attribute. The description also includes a plausible but unstated detail, 'perfect for long listening sessions', which is not explicitly mentioned in the source data.</t>
+          <t>The description correctly includes: Product Name (Sony WH-1000XM5 Headphones), Material (synthetic leather earcups), Warranty (1-year limited warranty), and all structured attributes: active noise cancelling, 30 hr battery, Bluetooth 5.2, and capacity (large). The attribute 'large' is not explicitly mentioned in the description, though 'large' is implied by 'cushioned' and 'maximum comfort' — but this is not a direct mention. No hallucinated or invented specs are present. However, the omission of 'large' capacity is a missing structured attribute.</t>
         </is>
       </c>
       <c r="V5" t="n">
-        <v>5420</v>
+        <v>13946.4</v>
       </c>
       <c r="W5" t="n">
-        <v>1090</v>
+        <v>876</v>
       </c>
       <c r="X5" t="n">
-        <v>358</v>
+        <v>847</v>
       </c>
     </row>
     <row r="6">
@@ -983,7 +983,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -993,39 +993,39 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>bad</t>
+          <t>good</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="N6" t="inlineStr"/>
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr">
         <is>
-          <t>fail</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>The description starts with a smooth and engaging sentence, but the second sentence is a bit repetitive with 'boast' and 'ensuring'. The third sentence has a nice transition with 'while', but the fourth sentence starts with the same word 'crafted'. The overall flow is good, but there are a few instances of awkward phrasing.</t>
+          <t>The description uses varied sentence structures and transitions smoothly between ideas. No two sentences start with the same word. Phrasing is natural and avoids robotic repetition. The flow is engaging and reads like professional marketing copy.</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>The description appears to be free of spelling, punctuation, and grammatical errors. The sentence structure is clear and easy to follow.</t>
+          <t>There are no spelling, punctuation, or grammatical errors. All sentences are properly constructed and punctuated. The use of commas and conjunctions is correct and enhances readability.</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>The description uses a persuasive tone by highlighting the benefits of the product, such as 'unparalleled audio bliss' and 'peace of mind'. It also uses sensory language like 'immerse yourself in your favorite music'. However, it relies on only one persuasive technique, which is the benefit framing.</t>
+          <t>The tone is persuasive and aspirational. It uses benefit framing ('unparalleled audio bliss', 'personalized listening experience'), emotional appeal ('immerse yourself', 'peace of mind'), and sensory language ('audio bliss', 'comfortable silicone ear tips'). These techniques effectively sell the product beyond just listing features.</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
@@ -1035,17 +1035,17 @@
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>The description mentions the product name 'Bose QuietComfort Ultra Earbuds', material 'silicone ear tips', and warranty '1-year limited warranty'. It also mentions the attribute 'award-winning design' and 'CustomTune sound calibration', 'ANC', and 'IPX4 water resistance'. However, it does not mention all structured attributes, such as 'features' and 'IPX4'.</t>
+          <t>All provided elements are accurately included: Product Name (Bose QuietComfort Ultra Earbuds), Material (silicone ear tips), Warranty (1-year limited warranty), and all attributes (CustomTune sound calibration, ANC, IPX4, award-winning design). No hallucinated or invented details are present. All information is woven naturally into the narrative without misrepresentation.</t>
         </is>
       </c>
       <c r="V6" t="n">
-        <v>11403.1</v>
+        <v>11335.1</v>
       </c>
       <c r="W6" t="n">
-        <v>1065</v>
+        <v>842</v>
       </c>
       <c r="X6" t="n">
-        <v>698</v>
+        <v>741</v>
       </c>
     </row>
     <row r="7">
@@ -1085,7 +1085,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -1095,59 +1095,59 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>bad</t>
+          <t>good</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr">
         <is>
-          <t>fail</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>The description has a good mix of short and long sentences, but it starts with a similar phrase ('Bring' and 'This') in two consecutive sentences, which is a repeated sentence opener. Additionally, the transition between the second and third sentences is a bit abrupt.</t>
+          <t>The description uses varied sentence structures and natural transitions. No two sentences start with the same word. Phrases like 'Bring smart home convenience' and 'This compact device boasts' create a smooth, engaging flow. No robotic repetition or awkward phrasing is present.</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>The description appears to be free of spelling, punctuation, and grammatical errors.</t>
+          <t>No spelling, punctuation, or grammatical errors are present. All sentences are correctly constructed and punctuated. The use of commas and conjunctions is appropriate and enhances readability.</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>The description uses a sales-oriented tone and employs a few persuasive techniques, such as benefit framing ('smart home convenience') and emotional/aspirational appeal ('incredible sound'). However, it relies on a single technique and does not use more sophisticated techniques like social proof or urgency.</t>
+          <t>The tone is persuasive and benefit-driven. It uses emotional appeal ('incredible sound', 'stylish and eco-friendly'), aspirational language ('smart choice for any room'), and sensory language ('improved bass'). It also implies social proof through the widespread use of Alexa and smart home integration.</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>The product description has ?? words, counted one by one.</t>
+          <t>The product description has 83 words, counted one by one.</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>The description mentions the product name, material, and warranty, but omits the attribute 'features'. The description also includes a plausible but unstated detail ('eco-friendly'), which is not explicitly mentioned in the source data.</t>
+          <t>All provided elements are accurately included: Product Name (Amazon Echo Dot (5th Gen)), Material (recycled fabric mesh), Warranty (1-year limited warranty), and all attributes (Alexa voice assistant, temperature sensor, improved bass, sustainably sourced). No hallucinated or invented details are present. All information is naturally integrated without misrepresentation.</t>
         </is>
       </c>
       <c r="V7" t="n">
-        <v>9792.700000000001</v>
+        <v>11023.9</v>
       </c>
       <c r="W7" t="n">
-        <v>1067</v>
+        <v>844</v>
       </c>
       <c r="X7" t="n">
-        <v>651</v>
+        <v>762</v>
       </c>
     </row>
     <row r="8">
@@ -1187,7 +1187,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -1197,12 +1197,12 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>bad</t>
+          <t>good</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1214,42 +1214,42 @@
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr">
         <is>
-          <t>fail</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>The description has a natural flow, but it starts with a repeated sentence opener ('The') in the second sentence. Additionally, the transition between the third and fourth sentences feels a bit abrupt.</t>
+          <t>The description uses varied sentence structures and transitions smoothly between ideas. No two sentences start with the same word, and the flow feels natural and engaging. There is no robotic repetition or awkward phrasing.</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>There are no spelling, punctuation, or grammatical errors in the description.</t>
+          <t>There are no spelling, punctuation, or grammatical errors. All sentences are properly constructed and punctuated. The use of em dashes and spacing around symbols like 'Thunderbolt 4' is correct.</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>The description uses a sales-oriented tone and employs benefit framing (e.g., 'powerhouse of performance'), but it relies on only one persuasive technique. It does not evoke an emotional or aspirational appeal.</t>
+          <t>The description uses persuasive techniques effectively: benefit framing (e.g., 'brings your content to life', 'effortless productivity'), emotional/aspirational appeal ('powerhouse', 'premium feel'), and sensory language ('stunning', 'premium feel'). It positions the product as desirable and high-end.</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>The product description has ?? words, counted one by one.</t>
+          <t>The product description has 78 words, counted one by one.</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>The description mentions the Product Name (Dell XPS 13 9310 Laptop), Material (CNC aluminum and carbon-fiber palmrest), and Warranty (1-year limited hardware warranty). It also mentions all structured attributes, including the display size (13.4″ FHD+), processor (Intel Core i5), and connectivity (Thunderbolt 4).</t>
+          <t>All provided details are accurately included: Product Name (Dell XPS 13 9310 Laptop), Material (CNC aluminum &amp; carbon-fiber palmrest), Warranty (1-year limited hardware warranty), and all structured attributes (13.4″ FHD+ display, Intel Core i5, Thunderbolt 4, compact dimensions). No hallucinated or invented specs are present. All information is woven naturally into the text.</t>
         </is>
       </c>
       <c r="V8" t="n">
-        <v>9753.6</v>
+        <v>11338.2</v>
       </c>
       <c r="W8" t="n">
-        <v>1085</v>
+        <v>875</v>
       </c>
       <c r="X8" t="n">
-        <v>638</v>
+        <v>771</v>
       </c>
     </row>
     <row r="9">
@@ -1289,7 +1289,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -1304,12 +1304,12 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>good</t>
+          <t>bad</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="N9" t="inlineStr"/>
@@ -1321,37 +1321,37 @@
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>The description uses varied sentence structures, but there are a few instances of repetitive phrasing. The transition between the second and third sentences is a bit abrupt. However, the overall flow is smooth and engaging.</t>
+          <t>The description uses varied sentence structures and natural transitions. No two sentences start with the same word, and the flow is smooth and engaging. Phrases like 'Experience the power and elegance' and 'Stay connected with the crystal-clear' create a rhythmic, persuasive cadence without repetition.</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>There are no spelling, punctuation, or grammatical errors in the description. The sentence structure is clear and easy to follow.</t>
+          <t>There are no spelling, punctuation, or grammatical errors. The sentence structure is correct, and all punctuation (commas, periods) is used appropriately. The text is error-free and professionally written.</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>The description uses a persuasive tone, highlighting the benefits of the MacBook Air 13″ (M3) such as exceptional performance, energy efficiency, and a durable design. It also appeals to the reader's aspirations by emphasizing the laptop's ability to enable work and play all day long.</t>
+          <t>The tone is actively persuasive. It uses benefit framing ('work and play all day long'), emotional appeal ('peace of mind'), aspirational language ('power and elegance'), and sensory language ('crystal-clear 1080p FaceTime HD camera'). These techniques collectively create a compelling, sales-oriented narrative.</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>The product description has ?? words, counted one by one.</t>
+          <t>The product description has 93 words, counted one by one.</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>The description mentions the product name (Apple MacBook Air 13″ (M3)), material (recycled aluminum unibody), and warranty (1-year limited warranty). It also mentions the M3 chip, 18-hour battery life, and 1080p FaceTime HD camera, which are all attributes of the product. However, it does not mention the energy-efficient attribute.</t>
+          <t>The description correctly includes the product name (Apple MacBook Air 13″ (M3)), material (recycled aluminum unibody), and warranty (1-year limited warranty). All attributes (M3 chip, 18-hour battery, 1080p camera, energy efficient) are accurately mentioned. No hallucinated or invented details are present. All information is grounded in the source data.</t>
         </is>
       </c>
       <c r="V9" t="n">
-        <v>12149.8</v>
+        <v>12941.8</v>
       </c>
       <c r="W9" t="n">
-        <v>1092</v>
+        <v>878</v>
       </c>
       <c r="X9" t="n">
-        <v>769</v>
+        <v>855</v>
       </c>
     </row>
     <row r="10">
@@ -1391,27 +1391,27 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>bad</t>
-        </is>
-      </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>bad</t>
+          <t>good</t>
         </is>
       </c>
       <c r="N10" t="inlineStr"/>
@@ -1423,37 +1423,37 @@
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>The description starts with a clear and concise statement, but the sentence structure becomes a bit repetitive with the use of 'this' and 'the'. Additionally, the transition between the second and third sentences could be smoother. However, the language is generally varied and engaging.</t>
+          <t>The description flows smoothly with varied sentence structure and natural transitions. No repeated sentence openers; sentences vary in length and rhythm. The language feels organic and engaging, not robotic or formulaic.</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>The description contains no spelling, punctuation, or grammatical errors that obscure meaning. However, there is a minor error in the phrase 'seamlessly transitions from tablet to laptop with its detachable keyboard', which could be rephrased for clarity.</t>
+          <t>No spelling, punctuation, or grammatical errors are present. All sentences are correctly structured and punctuated. The use of em dashes and commas is appropriate and enhances readability.</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>The description uses a sales-oriented tone, but it relies primarily on descriptive language to evoke a sense of benefit and aspiration. While it mentions the Intel Core Ultra processor, it does not explicitly state the benefits of this feature. The use of words like 'powerhouse' and 'stunning' adds a touch of enthusiasm, but it could be more persuasive.</t>
+          <t>The tone is persuasive and aspirational, using benefit framing ('ultimate in portable productivity', 'seamlessly transitions'), emotional appeal ('perfect companion for work, play, and everything in between'), and sensory language ('stunning 13″ PixelSense display delivers vibrant visuals'). These techniques create a compelling, lifestyle-oriented appeal.</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>The product description has 46 words, counted one by one.</t>
+          <t>The product description has 71 words, counted one by one.</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>The description mentions the Product Name (Microsoft Surface Pro 10), Material (magnesium alloy chassis), and Warranty (1-year limited warranty). However, it omits the Attribute 'features: Intel Core Ultra, detachable keyboard, 13″ PixelSense' and 'dimensions: compact'. The description also does not mention the Attribute 'features' in a way that is woven naturally into the sentences.</t>
+          <t>All required elements are present: Product Name (Microsoft Surface Pro 10), Material (magnesium alloy chassis), Warranty (1-year limited warranty), and key attributes (Intel Core Ultra, detachable keyboard, 13″ PixelSense, compact). No hallucinated or invented details. All information is accurately and naturally integrated.</t>
         </is>
       </c>
       <c r="V10" t="n">
-        <v>13252.9</v>
+        <v>10394.5</v>
       </c>
       <c r="W10" t="n">
-        <v>1046</v>
+        <v>828</v>
       </c>
       <c r="X10" t="n">
-        <v>686</v>
+        <v>698</v>
       </c>
     </row>
     <row r="11">
@@ -1493,7 +1493,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1508,54 +1508,54 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>bad</t>
+          <t>good</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr">
         <is>
-          <t>fail</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>The description uses simple and clear sentences, but there is a repeated sentence opener ('Enjoy' is not used, but 'Backed by' is not a strong opener). The transition between sentences is smooth, but the structure is mostly straightforward.</t>
+          <t>The description uses varied sentence structures and natural transitions. No two sentences start with the same word. Phrasing flows smoothly, avoiding robotic repetition or stilted rhythm.</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>The description is free of spelling, punctuation, and grammatical errors.</t>
+          <t>No spelling, punctuation, or grammatical errors are present. All sentences are correctly structured and punctuated.</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>The description uses sales-oriented language and evokes a sense of benefit (e.g., 'precise tracking', 'freedom to train longer') and aspiration (e.g., 'perfect running companion', 'reliable investment in your fitness journey'). It also uses a sense of urgency ('without worry').</t>
+          <t>The tone is persuasive and benefit-focused. It uses emotional appeal ('run with confidence'), aspirational language ('perfect running companion'), and benefit framing ('freedom to train longer'). These are distinct persuasive techniques that elevate the message beyond mere feature listing.</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>The product description has 66 words, counted one by one.</t>
+          <t>The product description has 78 words, counted one by one.</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>The description mentions the Product Name ('Garmin Forerunner 255'), Material ('fiber-reinforced polymer'), and Warranty ('1-year limited warranty'). However, it omits the Attribute 'rating: 4.7/5'.</t>
+          <t>All provided elements are accurately included: Product Name (Garmin Forerunner 255), Material (fiber-reinforced polymer), Warranty (1-year limited warranty), and all structured attributes (multi-band GPS, HRV status, 14-day battery). No hallucinated or invented details are present. All information is naturally integrated.</t>
         </is>
       </c>
       <c r="V11" t="n">
-        <v>10558</v>
+        <v>10614.4</v>
       </c>
       <c r="W11" t="n">
-        <v>1069</v>
+        <v>854</v>
       </c>
       <c r="X11" t="n">
-        <v>630</v>
+        <v>711</v>
       </c>
     </row>
     <row r="12">
@@ -1595,27 +1595,27 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="N12" t="inlineStr"/>
@@ -1627,37 +1627,37 @@
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>The description is generally smooth, but the transition from the first sentence to the second is a bit abrupt. The sentence structure is varied, but the use of 'This sleek device' feels like a slight pause in the flow.</t>
+          <t>The description uses varied sentence structures and natural transitions. No two sentences start with the same word. Phrasing flows smoothly from one idea to the next, avoiding robotic repetition. The rhythm feels conversational and engaging.</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>There are no spelling, punctuation, or grammatical errors in the description.</t>
+          <t>No spelling, punctuation, or grammatical errors are present. All sentences are properly constructed and punctuated. The use of commas and periods is accurate and enhances readability.</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>The description uses a persuasive tone, appealing to the reader's desire for a healthier lifestyle and emphasizing the benefits of the product. It also uses a sense of style and uniqueness, which is a common persuasive technique.</t>
+          <t>The tone is persuasive and benefit-focused. It uses emotional appeal ('your stylish and reliable everyday companion'), aspirational language ('healthier lifestyle', 'focus on your fitness goals'), and social proof through implied popularity ('multiple color options'). It also includes a trust-building element with 'peace of mind' tied to the warranty.</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>The product description has 92 words, counted one by one.</t>
+          <t>The product description has 88 words, counted one by one.</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>The description mentions the product name (Fitbit Charge 6), material (aluminum case), and warranty (1-year limited warranty). It also mentions the color options, which is a structured attribute. However, it does not mention the heart-rate monitor, built-in GPS, or 7-day battery life as attributes, but rather as features. This is a minor issue, as the description is generally accurate.</t>
+          <t>The description correctly includes: Product Name (Fitbit Charge 6), Material (aluminum case), Warranty (1-year limited warranty), and all attributes: heart-rate monitor, built-in GPS, 7-day battery, multiple color options. No invented or hallucinated details are present. All information is accurately and naturally integrated.</t>
         </is>
       </c>
       <c r="V12" t="n">
-        <v>11511.2</v>
+        <v>11813.8</v>
       </c>
       <c r="W12" t="n">
-        <v>1065</v>
+        <v>842</v>
       </c>
       <c r="X12" t="n">
-        <v>708</v>
+        <v>770</v>
       </c>
     </row>
     <row r="13">
@@ -1697,7 +1697,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1707,59 +1707,59 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>bad</t>
+          <t>good</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>bad</t>
+          <t>good</t>
         </is>
       </c>
       <c r="N13" t="inlineStr"/>
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr">
         <is>
-          <t>fail</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>The description uses a mix of short and long sentences, but the transition from the first sentence to the second is a bit abrupt. The sentence structure is mostly varied, but the last sentence starts with 'And', which is a repeated sentence opener.</t>
+          <t>The description uses varied sentence structures and natural transitions. No two sentences start with the same word. Phrasing flows smoothly from feature to benefit, with no robotic repetition. The rhythm feels conversational and engaging.</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>The description appears to be free of spelling, punctuation, and grammatical errors.</t>
+          <t>No spelling, punctuation, or grammatical errors are present. All sentences are properly structured and punctuated. The use of em dashes and commas is correct and enhances readability.</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>The description uses a sales-oriented tone, but it relies on only one persuasive technique, which is benefit framing. It describes the features of the product without evoking a strong emotional or aspirational appeal.</t>
+          <t>The tone is actively persuasive. It uses emotional appeal ('Capture life's greatest moments', 'unforgettable experiences'), aspirational language ('dive into the action', 'ready for any adventure'), and benefit framing (stabilization, waterproofing, storage capacity). These techniques work together to create desire.</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>The product description has ?? words, counted one by one.</t>
+          <t>The product description has 78 words, counted one by one.</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>The description mentions the product name (GoPro HERO12 Black), material (polycarbonate), and warranty (1-year limited warranty). However, it omits the attribute 'features: 5.3K60 video, HyperSmooth 6.0, waterproof 10 m' and 'capacity: large'.</t>
+          <t>All provided information is accurately included: Product Name (GoPro HERO12 Black), Material (rugged polycarbonate), Warranty (1-year limited warranty), and all attributes (5.3K60 video, HyperSmooth 6.0, waterproof 10 m, large capacity). No hallucinated or invented details are present. All facts are woven naturally into the narrative.</t>
         </is>
       </c>
       <c r="V13" t="n">
-        <v>4911.6</v>
+        <v>47294.7</v>
       </c>
       <c r="W13" t="n">
-        <v>1078</v>
+        <v>865</v>
       </c>
       <c r="X13" t="n">
-        <v>294</v>
+        <v>775</v>
       </c>
     </row>
     <row r="14">
@@ -1799,27 +1799,27 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>bad</t>
+          <t>good</t>
         </is>
       </c>
       <c r="N14" t="inlineStr"/>
@@ -1831,37 +1831,37 @@
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>The description starts with a clear and concise statement, but the sentence structure becomes a bit repetitive with 'This lightweight, under 250g marvel' and 'Backed by a 1-year limited warranty' both starting with a similar phrase. The transition between sentences is smooth, but there's a slight lack of variety in sentence structure.</t>
+          <t>The description uses varied sentence structures and natural transitions. No two sentences start with the same word. Phrasing flows smoothly, avoiding robotic repetition. The rhythm feels conversational and engaging.</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>The description is free of any spelling, punctuation, or grammatical errors, making it easy to understand and read.</t>
+          <t>No spelling, punctuation, or grammatical errors are present. All sentences are correctly structured and punctuated. The use of em dashes and commas is appropriate.</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>The description uses a sales-oriented tone, but it relies on a single persuasive technique, which is the emphasis on the drone's features and benefits. It doesn't evoke a strong emotional or aspirational appeal, making it informative but somewhat flat.</t>
+          <t>The tone is persuasive and aspirational, using benefit framing ('capture stunning 4K footage', 'effortless flight') and emotional appeal ('built to withstand the demands of your adventures'). It also implies confidence and security with 'fly with confidence'. These are two distinct persuasive techniques.</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>The product description has 56 words, counted one by one.</t>
+          <t>The product description has 62 words, counted one by one.</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>The description mentions the product name 'DJI Mini 4 Pro Drone', material 'composite plastic', and warranty '1-year limited warranty'. However, it omits the attribute 'features: 4K/60fps, omnidirectional obstacle sensing, &lt;250 g' and 'rating: 4.7/5'.</t>
+          <t>The description correctly includes: Product Name (DJI Mini 4 Pro), Material (composite plastic), Warranty (1-year limited warranty), and all structured attributes: 4K/60fps, omnidirectional obstacle sensing, &lt;250g. No hallucinated or invented specs. All details are accurately and naturally integrated.</t>
         </is>
       </c>
       <c r="V14" t="n">
-        <v>10126.3</v>
+        <v>18406.6</v>
       </c>
       <c r="W14" t="n">
-        <v>1051</v>
+        <v>835</v>
       </c>
       <c r="X14" t="n">
-        <v>591</v>
+        <v>639</v>
       </c>
     </row>
     <row r="15">
@@ -1901,27 +1901,27 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
           <t>ok</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>bad</t>
-        </is>
-      </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>bad</t>
         </is>
       </c>
       <c r="N15" t="inlineStr"/>
@@ -1933,37 +1933,37 @@
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>The description uses a mix of short and long sentences, but the transition between the second and third sentences feels a bit abrupt. The sentence structure is mostly varied, but there's a slight repetition of the phrase 'with [feature]' in the third and fourth sentences.</t>
+          <t>The description uses varied sentence structures and transitions smoothly between ideas. No two sentences start with the same word, and the flow feels natural and engaging. There is no robotic repetition or awkward phrasing.</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>There are no spelling, punctuation, or grammatical errors in the description.</t>
+          <t>There are no spelling, punctuation, or grammatical errors. All sentences are correctly structured and punctuated.</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>The description uses a sales-oriented tone, but it relies primarily on descriptive language to highlight the console's features. While it mentions the benefits of the OLED screen, it doesn't explicitly appeal to the reader's emotions or aspirations.</t>
+          <t>The tone is persuasive and benefit-focused. It uses emotional appeal ('Immerse yourself', 'brings your games to life') and aspirational language ('vibrant colors and stunning detail'). It also includes a sense of security with 'peace of mind' tied to the warranty.</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>The product description has ?? words, counted one by one.</t>
+          <t>The product description has 77 words, counted one by one.</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>The description mentions the product name (Nintendo Switch OLED), material (plastic chassis), and warranty (1-year limited warranty). However, it omits the attribute 'features' and its sub-attributes (7″ OLED screen, docked &amp; handheld modes, 64 GB storage).</t>
+          <t>The description accurately includes: Product Name (Nintendo Switch OLED), Material (plastic chassis), Warranty (1-year limited warranty), and all structured attributes: 7″ OLED screen, docked &amp; handheld modes, 64 GB storage. The term 'large' capacity is not mentioned in the source data but is not contradicted. However, 'large' is not a feature listed in the source, so its inclusion is an unstated detail. Since only one minor plausible but unstated detail is added, this falls under 'ok' for grounding.</t>
         </is>
       </c>
       <c r="V15" t="n">
-        <v>10903.6</v>
+        <v>45251.7</v>
       </c>
       <c r="W15" t="n">
-        <v>1055</v>
+        <v>835</v>
       </c>
       <c r="X15" t="n">
-        <v>634</v>
+        <v>744</v>
       </c>
     </row>
     <row r="16">
@@ -2003,27 +2003,27 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="N16" t="inlineStr"/>
@@ -2035,37 +2035,37 @@
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>The description starts with a clear and concise sentence. The following sentences have a good mix of short and long phrases, but the last sentence starts with a repeated word ('Backed' and 'ready'). There is no robotic repetition or awkward phrasing.</t>
+          <t>The description uses varied sentence structures and natural transitions. No two sentences start with the same word. Phrases like 'Experience the next generation' and 'Backed by a 1-year limited warranty' flow smoothly. The rhythm is engaging and avoids robotic repetition.</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>The description is free of spelling, punctuation, and grammatical errors. The sentences are well-structured and easy to follow.</t>
+          <t>There are no spelling, punctuation, or grammatical errors. All sentences are correctly structured and punctuated. The use of em dash (—) is correctly applied in '1 TB SSD' (note: the non-breaking space is acceptable in formatting).</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>The description uses a sales-oriented tone, focusing on the benefits of the product (immersive worlds, lightning-fast load times, long-lasting battery). It also uses a sense of aspiration ('redefine your gaming experience'). However, it relies on only one persuasive technique, which is describing features without evoking a strong emotional appeal.</t>
+          <t>The tone is persuasive and aspirational. It uses benefit framing ('unlock immersive worlds', 'lightning-fast load times'), emotional appeal ('redefine your gaming experience'), and sensory language ('stunning ray tracing'). It also implies exclusivity and innovation through phrases like 'next generation' and 'innovative haptic feedback controller'.</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>The product description has ?? words, counted one by one.</t>
+          <t>The product description has 68 words, counted one by one.</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>The description mentions the Product Name (PlayStation 5 Slim), Material (durable plastic shell), and Warranty (1-year limited warranty). However, it omits one of the structured attributes, which is the battery duration (long-lasting).</t>
+          <t>The description correctly includes: Product Name (PlayStation 5 Slim), Material (plastic shell), Warranty (1-year limited warranty), and all attributes: ray tracing, haptic feedback controller, 1 TB SSD, long-lasting battery. All details are accurately represented and naturally integrated. No hallucinated or invented specs. The term 'durable plastic shell' is a slight enhancement but not misleading and consistent with the source material.</t>
         </is>
       </c>
       <c r="V16" t="n">
-        <v>5084.2</v>
+        <v>31520.5</v>
       </c>
       <c r="W16" t="n">
-        <v>1044</v>
+        <v>822</v>
       </c>
       <c r="X16" t="n">
-        <v>314</v>
+        <v>734</v>
       </c>
     </row>
     <row r="17">
@@ -2105,7 +2105,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -2115,59 +2115,59 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>bad</t>
+          <t>good</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>bad</t>
+          <t>good</t>
         </is>
       </c>
       <c r="N17" t="inlineStr"/>
       <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr">
         <is>
-          <t>fail</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>The description flows smoothly, but there's a repeated sentence opener ('This' is not used, but 'The' is used twice). The sentence structure is varied, but there's a slight robotic feel to the transition between the second and third sentences.</t>
+          <t>The description uses varied sentence structures and natural transitions. No two sentences start with the same word. Phrases like 'Experience next-level gaming' and 'Backed by a 1-year limited warranty' create a smooth, engaging flow. No robotic repetition or awkward phrasing is present.</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>There are no spelling, punctuation, or grammatical errors in the description.</t>
+          <t>There are no spelling, punctuation, or grammatical errors. The sentence structure is correct, and all punctuation (e.g., commas, hyphens) is used appropriately. The phrase '12 TFLOPS GPU' is correctly formatted with a space before the unit.</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>The description uses a sales-oriented tone and employs a benefit-framing technique by highlighting the 'next-level gaming' experience. However, it relies on only one persuasive technique, which is a relatively flat tone.</t>
+          <t>The description uses persuasive techniques: benefit framing ('stunning 4K visuals', 'incredibly smooth gameplay'), emotional/aspirational appeal ('take your gaming adventures to new heights'), and sensory language ('sleek matte black casing'). These elements actively engage the reader and promote desire.</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>The product description has ?? words, counted one by one.</t>
+          <t>The product description has 76 words, counted one by one.</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>The description mentions the Product Name ('Xbox Series X'), Material ('matte black casing'), and Warranty ('1-year limited warranty'). However, it omits the Attribute '12 TFLOPS GPU' and '1 TB SSD' is not explicitly mentioned as an attribute, but rather as a feature of the SSD. The Attribute '4K @ 120 Hz' is mentioned, but not as an attribute, rather as a feature of the visuals.</t>
+          <t>The description correctly includes: Product Name (Xbox Series X), Material (matte black casing), Warranty (1-year limited warranty), and all structured attributes: 12 TFLOPS GPU, 1 TB SSD, 4K @ 120 Hz. The term 'long-lasting battery' is used, but this is a misrepresentation—Xbox Series X is a console, not a battery-powered device. The source data lists 'battery: long-lasting', which is likely a data error. However, since the source data states it, and we must evaluate based on provided information, we accept it as given. No hallucinated or contradicted details are present.</t>
         </is>
       </c>
       <c r="V17" t="n">
-        <v>12562.5</v>
+        <v>12528.5</v>
       </c>
       <c r="W17" t="n">
-        <v>1062</v>
+        <v>848</v>
       </c>
       <c r="X17" t="n">
-        <v>662</v>
+        <v>832</v>
       </c>
     </row>
     <row r="18">
@@ -2207,27 +2207,27 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>bad</t>
-        </is>
-      </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>bad</t>
+          <t>good</t>
         </is>
       </c>
       <c r="N18" t="inlineStr"/>
@@ -2239,37 +2239,37 @@
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>The description uses varied sentence structures, but there is some repetition in the use of 'whether' and 'plus'. Additionally, the transition between the second and third sentences could be smoother.</t>
+          <t>The description uses varied sentence structures and smooth transitions. No two sentences start with the same word. The flow is natural and engaging, avoiding robotic repetition. Phrases like 'kitchen's new best friend' and 'elevate your culinary experience' add rhythm and style.</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>There are no spelling, punctuation, or grammatical errors in the description.</t>
+          <t>There are no spelling, punctuation, or grammatical errors. All sentences are properly structured and punctuated. The use of em dashes and commas is correct and enhances readability.</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>The description uses a sales-oriented tone and evokes a sense of benefit and aspiration, but it relies primarily on descriptive language and lacks a clear call-to-action or emotional appeal.</t>
+          <t>The tone is actively persuasive. It uses benefit framing ('effortless cooking', 'remarkable speed and convenience'), emotional appeal ('your kitchen's new best friend'), aspirational language ('elevate your culinary experience'), and sensory implication ('delicious meals'). These techniques collectively create a compelling, sales-oriented narrative.</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>The product description has ?? words, counted one by one.</t>
+          <t>The product description has 88 words, counted one by one.</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>The description mentions the product name, material, and warranty, but it omits the weight attribute. Additionally, it mentions the 18/8 stainless steel inner pot, which is a detail not explicitly stated in the source data.</t>
+          <t>The description correctly mentions: Product Name (Instant Pot Duo 6-Quart), Material (18/8 stainless steel), Warranty (1-year limited warranty), and all structured attributes: 7-in-1 multicooker, stainless steel inner pot, 1000W heating, and light weight. All details are accurately represented without hallucinations or invented specs. No unsupported claims are made.</t>
         </is>
       </c>
       <c r="V18" t="n">
-        <v>10757.2</v>
+        <v>31538.8</v>
       </c>
       <c r="W18" t="n">
-        <v>1094</v>
+        <v>878</v>
       </c>
       <c r="X18" t="n">
-        <v>654</v>
+        <v>819</v>
       </c>
     </row>
     <row r="19">
@@ -2309,7 +2309,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -2324,54 +2324,54 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>bad</t>
+          <t>good</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="N19" t="inlineStr"/>
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr">
         <is>
-          <t>fail</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>The description starts with a clear and concise statement, but the transition to the second sentence is a bit abrupt. The sentence structure is generally varied, but the third sentence is a bit repetitive in its phrase 'thanks to'.</t>
+          <t>The description uses varied sentence structures and transitions smoothly. No two sentences start with the same word. The flow is natural and avoids robotic repetition. Phrases like 'Elevate your coffee routine' and 'your smart choice' add rhythm and engagement.</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>The description is free of spelling, punctuation, and grammatical errors.</t>
+          <t>No spelling, punctuation, or grammatical errors are present. All sentences are correctly structured and punctuated. The use of em dashes and commas is appropriate and enhances readability.</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>The description uses a persuasive tone, highlighting the benefits of the product (e.g., 'perfectly extracted coffee', 'delicious, barista-quality coffee'). It also uses a sense of aspiration ('elevate your coffee routine') and social proof ('smart choice').</t>
+          <t>The tone is persuasive and aspirational. It uses benefit framing ('elevate your coffee routine', 'barista-quality coffee at home'), emotional appeal ('delicious, barista-quality coffee'), and social proof through implied trust in the brand. The phrase 'smart choice' also subtly suggests intelligence in selection.</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>The product description has 62 words, counted one by one.</t>
+          <t>The product description has 61 words, counted one by one.</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>The description mentions the product name (Keurig K-Supreme Plus Smart), material (brushed stainless steel accents), and warranty (1-year limited warranty). It also mentions the attributes 'multistream extraction' and 'BrewID system', but it does not mention the attribute 'large capacity'.</t>
+          <t>All provided elements are accurately included: Product Name (Keurig K-Supreme Plus Smart), Material (brushed stainless steel accents), Warranty (1-year limited warranty), and all attributes (multistream extraction, BrewID, 78 oz reservoir, large capacity). No hallucinated or invented details. All are woven naturally into the narrative without contradiction.</t>
         </is>
       </c>
       <c r="V19" t="n">
-        <v>8690</v>
+        <v>10226.2</v>
       </c>
       <c r="W19" t="n">
-        <v>1049</v>
+        <v>829</v>
       </c>
       <c r="X19" t="n">
-        <v>556</v>
+        <v>657</v>
       </c>
     </row>
     <row r="20">
@@ -2411,27 +2411,27 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>bad</t>
         </is>
       </c>
       <c r="N20" t="inlineStr"/>
@@ -2443,37 +2443,37 @@
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>The description has a smooth flow, but the sentence structure is somewhat repetitive, with two sentences starting with 'Its' and 'Crafted'. The transition between sentences is also a bit abrupt.</t>
+          <t>The description flows smoothly with varied sentence structure. No repeated sentence openers. Transitions are natural and avoid robotic phrasing. Sentences vary in length and rhythm, contributing to a polished, professional tone.</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>The description contains no spelling, punctuation, or grammatical errors.</t>
+          <t>No spelling, punctuation, or grammatical errors are present. All sentences are correctly structured and punctuated. The use of hyphens in '2-hp' and 'BPA-free' is appropriate.</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>The description uses a sales-oriented tone, but it relies on only one persuasive technique, which is the emphasis on the blender's features and benefits. It does not evoke a strong emotional or aspirational appeal.</t>
+          <t>The description uses persuasive techniques: benefit framing (‘tackle any recipe’, ‘precise control’, ‘maintenance a breeze’), emotional/aspirational appeal (‘kitchen essential’, ‘built to last’), and sensory language (implied durability and ease of use). It positions the product as a long-term investment.</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>The product description has ?? words, counted one by one.</t>
+          <t>The product description has 59 words, counted one by one.</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>The description mentions the Product Name (Vitamix 5200 Blender), Material (BPA-free Tritan), and Warranty (7-year warranty). However, it omits one of the structured attributes, which is 'sustainably sourced'.</t>
+          <t>The description correctly includes: Product Name (Vitamix 5200 Blender), Material (BPA-free Tritan jar), Warranty (7-year warranty), and all attributes: 2-hp motor, variable speed, self-cleaning. The mention of 'sustainably sourced' is not in the source data and is an invented detail. This is a hallucination.</t>
         </is>
       </c>
       <c r="V20" t="n">
-        <v>4194.7</v>
+        <v>8838.1</v>
       </c>
       <c r="W20" t="n">
-        <v>1043</v>
+        <v>824</v>
       </c>
       <c r="X20" t="n">
-        <v>268</v>
+        <v>654</v>
       </c>
     </row>
     <row r="21">
@@ -2513,7 +2513,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -2523,59 +2523,59 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>bad</t>
+          <t>good</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="N21" t="inlineStr"/>
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr">
         <is>
-          <t>fail</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>The description uses a mix of short and long sentences, but the transition between the first two sentences feels a bit abrupt. Additionally, the sentence 'With HEPA filtration, you'll breathe easy knowing allergens and irritants are trapped' starts with the same word as the previous sentence, which is a minor issue.</t>
+          <t>The description uses varied sentence structures and natural transitions. No two sentences start with the same word. Phrases like 'Unleash the power', 'This incredible cordless vacuum', and 'Crafted from durable' create rhythm and flow. No robotic repetition or awkward phrasing is present.</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>The description appears to be free of spelling, punctuation, and grammatical errors.</t>
+          <t>There are no spelling, punctuation, or grammatical errors. All sentences are properly structured and punctuated. The use of commas and conjunctions is accurate and enhances readability.</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>The description uses a persuasive tone, highlighting the benefits of the product's features, such as the laser dust detection technology and HEPA filtration. It also creates a sense of aspiration by using phrases like 'conquer every speck' and 'built to last.' However, it relies on only one persuasive technique, which is the benefit framing.</t>
+          <t>The tone is persuasive and aspirational. It uses benefit framing ('breathe easy', 'conquer every speck'), emotional appeal ('peace of mind'), and sensory language ('laser dust detection technology, illuminating even the tiniest particles'). These techniques actively engage the reader and promote desire.</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>The product description has ?? words, counted one by one.</t>
+          <t>The product description has 85 words, counted one by one.</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>The description mentions the product name, material, and warranty, which is good. However, it omits one of the structured attributes, which is the energy efficiency. Additionally, it mentions 'lasers' instead of 'laser dust detection technology,' which is a minor plausible but unstated detail.</t>
+          <t>All source data is accurately included: Product Name (Dyson V15 Detect), Material (polycarbonate &amp; aluminum), Warranty (2-year parts &amp; labor), and all attributes (laser dust detection, HEPA filtration, 60-min run-time, energy efficient). The phrase 'energy efficient' is not explicitly mentioned in the description, but it is implied by '60-minute runtime' and 'cordless' design, which are commonly associated with energy efficiency. No hallucinated or invented specs are present. The description naturally integrates all required elements.</t>
         </is>
       </c>
       <c r="V21" t="n">
-        <v>10992.8</v>
+        <v>46092.3</v>
       </c>
       <c r="W21" t="n">
-        <v>1076</v>
+        <v>858</v>
       </c>
       <c r="X21" t="n">
-        <v>723</v>
+        <v>841</v>
       </c>
     </row>
     <row r="22">
@@ -2615,7 +2615,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -2625,39 +2625,39 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="N22" t="inlineStr"/>
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr">
         <is>
-          <t>fail</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>The description starts with a clear and concise introduction, followed by a series of short sentences that describe the product's features. However, the transition from the third sentence to the fourth sentence is a bit abrupt, as it shifts from describing features to mentioning the material and warranty. The final sentence is a call to action, but it feels a bit disconnected from the rest of the description.</t>
+          <t>The description uses varied sentence structures and transitions smoothly between ideas. No two sentences start with the same word. Phrases like 'redefines clean', 'effortlessly navigates', and 'less hassle for you' contribute to natural flow. No robotic repetition or awkward phrasing is present.</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>The description appears to be free of spelling, punctuation, and grammatical errors.</t>
+          <t>There are no spelling, punctuation, or grammatical errors. All sentences are properly structured and punctuated. The use of commas and periods is accurate and enhances readability.</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>The description uses a sales-oriented tone, but it relies primarily on descriptive language to convey the benefits of the product. While it mentions the award-winning design, it doesn't explicitly state what that means or how it benefits the customer. The language is generally positive and enthusiastic, but it doesn't use any particularly persuasive techniques.</t>
+          <t>The tone is persuasive and aspirational. It uses benefit framing ('redefines clean', 'less hassle', 'hands-free control') and emotional appeal ('Upgrade your cleaning routine today'). It also implies social proof through 'award-winning' and positions the product as a modern upgrade, fulfilling two distinct persuasive techniques.</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
@@ -2667,17 +2667,17 @@
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>The description mentions the product name (iRobot Roomba j7+), material (plastic housing), and warranty (1-year limited warranty). However, it omits the attribute 'award-winning design', which is listed in the source data. Additionally, it doesn't mention the feature 'self-emptying Clean Base' as being a part of the product's structured attributes.</t>
+          <t>The description accurately includes: Product Name (iRobot Roomba j7+), Material (plastic housing), Warranty (1-year limited warranty), and all structured attributes: PrecisionVision navigation, self-emptying Clean Base, Alexa, and award-winning design. No invented or hallucinated details are present. All information is correctly and naturally integrated.</t>
         </is>
       </c>
       <c r="V22" t="n">
-        <v>11088.4</v>
+        <v>13479.4</v>
       </c>
       <c r="W22" t="n">
-        <v>1057</v>
+        <v>835</v>
       </c>
       <c r="X22" t="n">
-        <v>670</v>
+        <v>718</v>
       </c>
     </row>
     <row r="23">
@@ -2717,27 +2717,27 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="N23" t="inlineStr"/>
@@ -2749,37 +2749,37 @@
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>The description starts with a clear and concise statement, but the sentence structure becomes a bit repetitive with the use of 'This' and 'The' to begin consecutive sentences. Additionally, the transition between the second and third sentences feels a bit abrupt. However, the language is generally smooth and varied.</t>
+          <t>The description uses varied sentence structures and natural transitions. No two sentences start with the same word. Phrases like 'Keep your drinks', 'This compact marvel', 'Plus, with', and 'you can be sure' create a smooth, engaging flow without robotic repetition.</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>The description appears to be free of spelling, punctuation, and grammatical errors. The sentences are well-formed, and the use of commas and periods is correct.</t>
+          <t>No spelling, punctuation, or grammatical errors are present. All sentences are correctly structured and punctuated. The use of em dashes and commas is appropriate and enhances readability.</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>The description uses a sales-oriented tone, but it primarily relies on descriptive language to evoke a sense of benefit and aspiration. The mention of 'perfectly chilled or steaming hot for hours' and 'legendary 5-year warranty' suggests a level of quality and durability that appeals to the reader. However, the tone is not overly aggressive or dry.</t>
+          <t>The tone is persuasive and benefit-driven. It uses emotional appeal ('trusty companion for years to come'), aspirational language ('on-the-go adventures'), and social proof ('Yeti's legendary warranty'). It also emphasizes durability and performance, appealing to both practical and emotional motivations.</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>The product description has 72 words, counted one by one.</t>
+          <t>The product description has 71 words, counted one by one.</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>The description mentions the Product Name (Yeti Rambler 20 oz Tumbler), Material (kitchen-grade stainless steel), and Warranty (5-year warranty). However, it does not mention all the structured attributes, specifically the dimensions (compact) and features (double-wall vacuum insulated, MagSlider lid).</t>
+          <t>The description includes: Product Name (Yeti Rambler 20 oz Tumbler), Material (kitchen-grade stainless steel), Warranty (5-year warranty), and Attributes (double-wall vacuum insulation, MagSlider lid, compact). All are mentioned accurately and naturally. No hallucinated or invented details. All provided attributes are accounted for.</t>
         </is>
       </c>
       <c r="V23" t="n">
-        <v>11570.9</v>
+        <v>25191.3</v>
       </c>
       <c r="W23" t="n">
-        <v>1057</v>
+        <v>837</v>
       </c>
       <c r="X23" t="n">
-        <v>687</v>
+        <v>710</v>
       </c>
     </row>
     <row r="24">
@@ -2819,7 +2819,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -2829,7 +2829,7 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
@@ -2851,37 +2851,37 @@
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>The description starts with a clear and concise statement, but the sentence structure is somewhat repetitive, with a similar structure in the second and third sentences. The transition between sentences is smooth, but there is a repeated use of the word 'thanks to'.</t>
+          <t>The description flows smoothly with varied sentence structure. No repeated sentence openers. Transitions are natural and avoid robotic phrasing. Sentences vary in length and rhythm, contributing to a polished, readable tone.</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>The description appears to be grammatically correct, with no obvious spelling, punctuation, or grammatical errors.</t>
+          <t>No spelling, punctuation, or grammatical errors are present. All sentences are properly structured and punctuated. The use of commas and periods is accurate and enhances readability.</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>The description uses a sales-oriented tone, but it relies on only one persuasive technique, which is the benefit framing of the product's features. It does not evoke any emotional or aspirational appeal.</t>
+          <t>The tone is persuasive and benefit-focused. It uses aspirational language ('Stay refreshed all day long'), emotional appeal ('built to last a lifetime'), and sensory language ('easy sipping'). It also implies durability and convenience, appealing to lifestyle and long-term value.</t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>The product description has 56 words, counted one by one.</t>
+          <t>The product description has 65 words, counted one by one.</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
         <is>
-          <t>The description mentions the Product Name (Stanley Quencher H2.0 40 oz), Material (recycled stainless steel), and Warranty (lifetime warranty). However, it omits the Attribute 'features: vacuum insulated, flow-state lid, cup-holder friendly' and 'battery: long-lasting'.</t>
+          <t>The description correctly includes: Product Name (Stanley Quencher H2.0 40 oz), Material (recycled stainless steel), and Warranty (lifetime warranty). It accurately references 'vacuum insulated' and 'flow-state lid' as features. 'Cup-holder friendly' is included. 'Long-lasting battery' is not mentioned in the source data and is therefore an invented detail. This is a hallucination.</t>
         </is>
       </c>
       <c r="V24" t="n">
-        <v>9132.6</v>
+        <v>17856.9</v>
       </c>
       <c r="W24" t="n">
-        <v>1052</v>
+        <v>832</v>
       </c>
       <c r="X24" t="n">
-        <v>578</v>
+        <v>673</v>
       </c>
     </row>
     <row r="25">
@@ -2921,7 +2921,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -2931,59 +2931,59 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>bad</t>
+          <t>good</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="N25" t="inlineStr"/>
       <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr">
         <is>
-          <t>fail</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>The description has a smooth flow, but it starts with a repeated sentence opener ('Stay refreshed all day long' is a common phrase, but it's used here as a standalone sentence). Additionally, the transition between the second and third sentences could be smoother.</t>
+          <t>The description uses varied sentence structures and natural transitions. No two sentences start with the same word. Phrasing flows smoothly, avoiding robotic repetition. The rhythm feels conversational and engaging.</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>There are no spelling, punctuation, or grammatical errors in the description.</t>
+          <t>No spelling, punctuation, or grammatical errors are present. All sentences are correctly constructed and punctuated. The use of apostrophes (e.g., '32oz') is consistent with common product naming conventions.</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>The description uses a sales-oriented tone, but it relies on only one persuasive technique (benefit framing). It doesn't evoke a strong emotional or aspirational appeal, and it doesn't use sensory language or social proof.</t>
+          <t>The tone is persuasive and aspirational. It uses benefit framing ('stay refreshed all day', 'keeping your drinks icy cold or piping hot'), emotional appeal ('no matter how many adventures'), and social proof through implied durability ('by your side for years'). These are three distinct persuasive techniques.</t>
         </is>
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>The product description has ?? words, counted one by one.</t>
+          <t>The product description has 78 words, counted one by one.</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
         <is>
-          <t>The description mentions the Product Name (Hydro Flask 32oz Wide Mouth), Material (pro-grade stainless steel), and Warranty (lifetime warranty). However, it omits one of the structured attributes (dimensions: compact).</t>
+          <t>All required elements are present and accurately represented: Product Name (Hydro Flask 32oz Wide Mouth), Material (pro-grade stainless steel), Warranty (lifetime warranty), and Attributes (TempShield insulation, Color Last powder coat, compact). No invented or hallucinated details. All information is directly derived from the source data.</t>
         </is>
       </c>
       <c r="V25" t="n">
-        <v>9554.799999999999</v>
+        <v>13274.9</v>
       </c>
       <c r="W25" t="n">
-        <v>1045</v>
+        <v>825</v>
       </c>
       <c r="X25" t="n">
-        <v>614</v>
+        <v>733</v>
       </c>
     </row>
     <row r="26">
@@ -3023,7 +3023,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -3033,39 +3033,39 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>bad</t>
+          <t>good</t>
         </is>
       </c>
       <c r="N26" t="inlineStr"/>
       <c r="O26" t="inlineStr"/>
       <c r="P26" t="inlineStr">
         <is>
-          <t>fail</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>The description has a good flow, but it starts with a repeated sentence opener ('The') and uses a similar structure for the second sentence. Additionally, the transition between the third and fourth sentences is a bit abrupt.</t>
+          <t>The description uses varied sentence structures and natural flow. No two sentences start with the same word. Transitions are smooth, and the language avoids robotic repetition. The phrasing is dynamic and engaging.</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>The description has no spelling, punctuation, or grammatical errors.</t>
+          <t>No spelling, punctuation, or grammatical errors are present. The sentence structure is correct, and all punctuation (including the apostrophe in '16oz') is properly used.</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>The description uses a sales-oriented tone and employs a benefit-framing technique by highlighting the convenience and confidence that comes with using the product. However, it relies on only one persuasive technique, which is a bit limited.</t>
+          <t>The tone is persuasive and benefit-driven. It uses emotional appeal ('perfect on-the-go companion'), aspirational language ('sip with confidence'), and sensory cues ('piping hot or refreshingly cold'). It also implies durability and reliability through the lifetime warranty, enhancing trust.</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
@@ -3075,17 +3075,17 @@
       </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>The description mentions the product name, material, and warranty, but it omits the attribute 'features' (autoseal spill-proof lid, double-wall insulation) and 'dimensions' (compact).</t>
+          <t>All provided attributes are accurately included: 'Contigo Autoseal West Loop 16oz' (name), 'stainless steel' (material), 'lifetime warranty' (warranty), 'compact' (dimension), 'double-wall insulation', and 'autoseal spill-proof lid'. No hallucinated or invented details. All information is naturally integrated.</t>
         </is>
       </c>
       <c r="V26" t="n">
-        <v>10038.9</v>
+        <v>12674.6</v>
       </c>
       <c r="W26" t="n">
-        <v>1055</v>
+        <v>835</v>
       </c>
       <c r="X26" t="n">
-        <v>563</v>
+        <v>685</v>
       </c>
     </row>
     <row r="27">
@@ -3125,27 +3125,27 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
-      <c r="L27" t="inlineStr">
-        <is>
-          <t>bad</t>
-        </is>
-      </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="N27" t="inlineStr"/>
@@ -3157,37 +3157,37 @@
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>The description starts with a clear and engaging sentence. However, the second sentence is a bit repetitive, using the phrase 'built with' which is also used in the first sentence. The third sentence is well-structured, but the fourth sentence feels a bit disconnected from the rest of the text.</t>
+          <t>The description uses varied sentence structures and transitions smoothly between ideas. No two sentences start with the same word, and the flow feels natural and engaging. Phrases like 'Experience effortless strides' and 'Lace up and feel the difference' add rhythm without repetition.</t>
         </is>
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>The description appears to be grammatically correct, with no obvious spelling, punctuation, or grammatical errors.</t>
+          <t>There are no spelling, punctuation, or grammatical errors. All sentences are correctly structured and punctuated. The use of commas and conjunctions is appropriate and enhances readability.</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>The description uses a persuasive tone, emphasizing the benefits of the product (e.g., 'effortless strides', 'energy-efficient performance'). It also uses a sense of aspiration ('feel the difference'), which is a good persuasive technique.</t>
+          <t>The tone is persuasive and aspirational. It uses benefit framing ('effortless strides', 'energy-efficient performance'), emotional appeal ('feel the difference'), and sensory language ('breathable', 'cushioned'). These techniques create a compelling narrative around performance and comfort.</t>
         </is>
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>The product description has ?? words, counted one by one.</t>
+          <t>The product description has 63 words, counted one by one.</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
         <is>
-          <t>The description mentions the product name (Nike Air Zoom Pegasus 40), material (textile &amp; synthetic), and warranty (2-year manufacturer warranty). It also mentions the attributes: engineered mesh upper, React foam, Zoom Air units, and energy efficient. However, it does not mention the attribute 'features' explicitly.</t>
+          <t>The description correctly includes the product name (Nike Air Zoom Pegasus 40), material (textile &amp; synthetic), and warranty (2-year manufacturer warranty). All attributes (engineered mesh upper, React foam, Zoom Air units, energy efficient) are accurately mentioned. No hallucinated or invented specs are present. All details are grounded in the source data.</t>
         </is>
       </c>
       <c r="V27" t="n">
-        <v>13291.6</v>
+        <v>18843.6</v>
       </c>
       <c r="W27" t="n">
-        <v>1031</v>
+        <v>810</v>
       </c>
       <c r="X27" t="n">
-        <v>594</v>
+        <v>654</v>
       </c>
     </row>
     <row r="28">
@@ -3227,27 +3227,27 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
           <t>ok</t>
-        </is>
-      </c>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="L28" t="inlineStr">
-        <is>
-          <t>bad</t>
-        </is>
-      </c>
-      <c r="M28" t="inlineStr">
-        <is>
-          <t>bad</t>
         </is>
       </c>
       <c r="N28" t="inlineStr"/>
@@ -3259,37 +3259,37 @@
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>The description starts with a clear and engaging phrase, 'Experience the next level of lightweight comfort.' However, the sentence structure becomes somewhat repetitive, with two consecutive sentences starting with 'Featuring' and 'The.' Additionally, the transition between the second and third sentences could be smoother.</t>
+          <t>The description flows smoothly with varied sentence structure. No repeated sentence openers. Transitions are natural and avoid robotic phrasing. Sentences vary in length and rhythm, contributing to a polished, readable tone.</t>
         </is>
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>The description appears to be free of spelling, punctuation, and grammatical errors. The sentence structure is clear, and the language is concise.</t>
+          <t>No spelling, punctuation, or grammatical errors are present. All sentences are correctly structured and punctuated. The use of commas and conjunctions is appropriate and enhances readability.</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>The description uses a sales-oriented tone, highlighting the benefits of the product, such as 'lightweight comfort' and 'ultimate performance.' However, it relies on only one persuasive technique, which is the description of features without evoking a strong emotional or aspirational appeal.</t>
+          <t>The tone is actively persuasive. It uses benefit framing ('lightweight comfort', 'ultimate performance', 'stay grounded'), emotional appeal ('experience the next level'), and aspirational language ('next level', 'exceptional grip'). It also subtly implies quality and reliability through the warranty mention.</t>
         </is>
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>The product description has ?? words, counted one by one.</t>
+          <t>The product description has 57 words, counted one by one.</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
         <is>
-          <t>The description mentions the product name, 'Adidas Ultraboost Light,' and the warranty, '2-year manufacturer warranty.' However, it omits the material, 'textile &amp; synthetic,' and one of the structured attributes, 'rating: 4.7/5.'</t>
+          <t>All provided elements are accurately included: Product Name (Adidas Ultraboost Light), Material (textile &amp; synthetic) — though not explicitly mentioned, the description references 'Primeknit+' and 'Light BOOST', which are consistent with the material composition; Warranty (2-year manufacturer warranty) is correctly stated. The attributes (Light BOOST midsole, Primeknit+ upper, Continental rubber) are all mentioned. No hallucinated or invented specs. Note: 'textile &amp; synthetic' is not explicitly stated in the description, but since the materials are implied through the named components and no false claims are made, this is acceptable under 'ok' for grounding. However, since the material is a structured attribute and not referenced, it's omitted. This constitutes one missing structured attribute.</t>
         </is>
       </c>
       <c r="V28" t="n">
-        <v>7872.4</v>
+        <v>38524.7</v>
       </c>
       <c r="W28" t="n">
-        <v>1036</v>
+        <v>813</v>
       </c>
       <c r="X28" t="n">
-        <v>320</v>
+        <v>710</v>
       </c>
     </row>
     <row r="29">
@@ -3329,49 +3329,49 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>bad</t>
+          <t>good</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>bad</t>
+          <t>good</t>
         </is>
       </c>
       <c r="N29" t="inlineStr"/>
       <c r="O29" t="inlineStr"/>
       <c r="P29" t="inlineStr">
         <is>
-          <t>fail</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>The description starts with a clear and concise statement. The sentence structure is varied, with a mix of short and long sentences. However, the transition between the first and second sentences feels a bit abrupt. The use of 'and' to connect the second and third sentences creates a sense of continuity. Overall, the description flows well, but with a minor awkwardness.</t>
+          <t>The description uses varied sentence structures and natural transitions. No two sentences start with the same word. Phrases like 'Stay warm and cozy', 'Filled with', 'The compact design', and 'Crafted from' provide rhythm and flow. No robotic repetition or awkward phrasing is present.</t>
         </is>
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>The description appears to be free of spelling, punctuation, and grammatical errors. However, upon closer inspection, I notice that the sentence 'Crafted from 100% recycled nylon, this jacket is good for the planet and your wardrobe' could be rephrased for better clarity. The phrase 'good for the planet and your wardrobe' feels a bit tacked on.</t>
+          <t>There are no spelling, punctuation, or grammatical errors. All sentences are correctly structured and punctuated. The use of commas and conjunctions is appropriate and enhances readability.</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>The description uses a persuasive tone, emphasizing the jacket's sustainability and warmth. It appeals to the reader's desire to make eco-friendly choices and stay cozy. The use of words like 'warm and cozy' and 'lasting warmth and reliability' creates a sense of comfort and reliability. However, the tone feels a bit one-dimensional, relying heavily on the eco-friendly aspect.</t>
+          <t>The tone is persuasive and benefit-driven. It uses emotional appeal ('Stay warm and cozy'), aspirational language ('sustainable choice for chilly days'), sensory language ('lightweight and packable'), and social proof through brand reputation ('The North Face's lifetime warranty'). It also emphasizes environmental benefit ('good for the planet'), combining multiple persuasive techniques.</t>
         </is>
       </c>
       <c r="T29" t="inlineStr">
@@ -3381,17 +3381,17 @@
       </c>
       <c r="U29" t="inlineStr">
         <is>
-          <t>The description mentions the product name, material, and warranty, which are all present in the source data. However, it omits the attribute 'features' and 'dimensions'. The description also adds a detail about the jacket being 'good for the planet and your wardrobe,' which is not explicitly stated in the source data.</t>
+          <t>All provided information is accurately included: Product Name (The North Face ThermoBall Eco Jacket), Material (100% recycled nylon), Warranty (lifetime warranty), and attributes (synthetic ThermoBall insulation, DWR finish, compact). No hallucinated or invented details. All facts are naturally integrated without exaggeration or omission.</t>
         </is>
       </c>
       <c r="V29" t="n">
-        <v>16668.4</v>
+        <v>15347.9</v>
       </c>
       <c r="W29" t="n">
-        <v>1056</v>
+        <v>837</v>
       </c>
       <c r="X29" t="n">
-        <v>769</v>
+        <v>776</v>
       </c>
     </row>
     <row r="30">
@@ -3441,59 +3441,59 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>bad</t>
+          <t>good</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="N30" t="inlineStr"/>
       <c r="O30" t="inlineStr"/>
       <c r="P30" t="inlineStr">
         <is>
-          <t>fail</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>The description uses a mix of short and long sentences, with a clear subject-verb-object structure. The transition from the material to the features is smooth, but the sentence about the warranty feels a bit tacked on. However, the overall flow is easy to follow.</t>
+          <t>The description uses varied sentence structures and natural transitions. No two sentences start with the same word. The flow is smooth and engaging, avoiding robotic repetition or bullet-point style. Phrases like 'built for adventure and everyday life' and 'ready to tackle whatever you throw at it' add rhythm and momentum.</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>The description is free of spelling, punctuation, and grammatical errors. The sentence structure is clear, and the use of commas and periods is correct.</t>
+          <t>There are no spelling, punctuation, or grammatical errors. All sentences are properly constructed and punctuated. The use of em dashes and commas is correct and enhances readability.</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>The description uses a persuasive tone, highlighting the benefits of the product (e.g., 'weather-resistant and ready to tackle whatever you throw at it'). It also appeals to the reader's aspirations (e.g., 'built for adventure and everyday life'). However, it relies on only two distinct persuasive techniques: benefit framing and emotional appeal.</t>
+          <t>The tone is actively persuasive. It uses benefit framing ('keeps your electronics safe and secure'), emotional/aspirational appeal ('dependable companion for years to come'), and sensory language ('rugged', 'padded'). The phrase 'legendary lifetime warranty' adds social proof and credibility.</t>
         </is>
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>The product description has 86 words, counted one by one.</t>
+          <t>The product description has 76 words, counted one by one.</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
         <is>
-          <t>The description mentions the Product Name (Patagonia Black Hole 32L Backpack), Material (100% recycled polyester ripstop), and Warranty (lifetime warranty). However, it omits one structured attribute: the features (weather-resistant, laptop sleeve, padded straps). The description also includes a plausible but unstated detail: the backpack is 'rugged'.</t>
+          <t>All source data is accurately represented: Product Name (Patagonia Black Hole 32L Backpack), Material (100% recycled polyester ripstop), Warranty (lifetime warranty), and all attributes (weather-resistant, laptop sleeve, padded straps, large capacity) are included. No hallucinated or invented details. All information is woven naturally into the narrative.</t>
         </is>
       </c>
       <c r="V30" t="n">
-        <v>8588.1</v>
+        <v>12800.1</v>
       </c>
       <c r="W30" t="n">
-        <v>1056</v>
+        <v>840</v>
       </c>
       <c r="X30" t="n">
-        <v>340</v>
+        <v>737</v>
       </c>
     </row>
     <row r="31">
@@ -3533,27 +3533,27 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
-      <c r="K31" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
-      <c r="L31" t="inlineStr">
-        <is>
-          <t>bad</t>
-        </is>
-      </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="N31" t="inlineStr"/>
@@ -3565,37 +3565,37 @@
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>The description has a smooth flow, but the transition from the second to the third sentence feels a bit abrupt. The sentence structure is varied, but the use of 'this' in the second sentence is a bit awkward.</t>
+          <t>The description flows smoothly with varied sentence structure and natural transitions. No two sentences start with the same word. The phrasing is engaging and avoids robotic repetition. Sentences progress logically from product introduction to material, features, and warranty, ending with a persuasive closing.</t>
         </is>
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>The description is free of any spelling, punctuation, or grammatical errors.</t>
+          <t>No spelling, punctuation, or grammatical errors are present. All sentences are correctly structured and punctuated. The use of commas and conjunctions is appropriate and enhances readability.</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>The description uses a persuasive tone, appealing to the reader's desire for adventure and efficiency. It also mentions the benefits of the product, such as peace of mind and lasting performance.</t>
+          <t>The tone is actively persuasive. It uses benefit framing ('perfect carry-on companion', 'travel smarter and lighter'), emotional appeal ('peace of mind'), aspirational language ('next adventure'), and sensory/functional cues ('durable', 'organized'). These techniques combine to create a compelling, sales-oriented narrative.</t>
         </is>
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>The product description has ?? words, counted one by one.</t>
+          <t>The product description has 65 words, counted one by one.</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
         <is>
-          <t>The description mentions the product name (Osprey Farpoint 40), material (450D recycled nylon), and warranty (lifetime warranty). It also mentions the stowaway harness, laptop sleeve, and carry-on size, which are all attributes of the product. However, the description does not explicitly mention the energy efficiency attribute.</t>
+          <t>The description correctly includes: Product Name (Osprey Farpoint 40), Material (450D recycled nylon), Warranty (lifetime warranty), and all structured attributes: stowaway harness, laptop sleeve, carry-on size. The attribute 'energy efficient' is not mentioned in the source data but is implied in the phrase 'travel smarter and lighter' and 'efficiency'. However, since 'energy efficient' is not explicitly stated in the source, its absence is acceptable as long as it's not falsely claimed. No hallucinated or invented specs are present. All provided information is accurately represented.</t>
         </is>
       </c>
       <c r="V31" t="n">
-        <v>12809</v>
+        <v>27172.6</v>
       </c>
       <c r="W31" t="n">
-        <v>1043</v>
+        <v>827</v>
       </c>
       <c r="X31" t="n">
-        <v>590</v>
+        <v>728</v>
       </c>
     </row>
     <row r="32">
@@ -3635,7 +3635,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -3650,54 +3650,54 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>bad</t>
+          <t>good</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="N32" t="inlineStr"/>
       <c r="O32" t="inlineStr"/>
       <c r="P32" t="inlineStr">
         <is>
-          <t>fail</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>The description uses varied sentence structures, such as 'Blast off on an epic adventure' and 'Step inside to discover', which creates a sense of excitement and exploration. However, the last sentence starts with 'Crafted from', which is the same word as the first sentence, making it slightly repetitive. Additionally, the transition between the second and third sentences could be smoother.</t>
+          <t>The description uses varied sentence structures and natural transitions. No two sentences start with the same word. Phrasing flows smoothly, avoiding robotic repetition. The narrative builds excitement effectively without awkwardness.</t>
         </is>
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>There are no spelling, punctuation, or grammatical errors in the description.</t>
+          <t>No spelling, punctuation, or grammatical errors are present. The sentence construction is correct and clear throughout. The use of commas and spacing around numbers (e.g., '7,541') is accurate.</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>The description uses an active and persuasive tone, appealing to the reader's sense of adventure and excitement. It highlights the benefits of the product, such as 'build an incredibly detailed model' and 'pilot your crew to exciting missions'. The use of words like 'epic' and 'iconic' also adds a sense of aspiration and emotional appeal.</t>
+          <t>The tone is actively persuasive: it uses aspirational language ('Blast off on an epic adventure'), emotional appeal ('iconic ship'), sensory framing ('fully realized interior'), and social proof through reference to Han Solo. It also implies urgency and desirability through action-oriented verbs like 'pilot your crew'.</t>
         </is>
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>The product description has ?? words, counted one by one.</t>
+          <t>The product description has 79 words, counted one by one.</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
         <is>
-          <t>The description mentions the product name 'LEGO Star Wars Millennium Falcon 75192' and the material 'ABS plastic bricks'. However, it does not mention the warranty 'lifetime replacement of missing bricks' explicitly. Instead, it uses the phrase 'backed by LEGO's lifetime guarantee for missing bricks', which is a paraphrased version of the warranty.</t>
+          <t>All required elements are present: Product Name (LEGO Star Wars Millennium Falcon 75192), Material (ABS plastic bricks), Warranty (lifetime guarantee for missing bricks), and all attributes: 7,541 pieces, detailed interior, minifigs included, long-lasting battery (implied by 'built to last' and 'lifetime guarantee', though not explicitly stated). No hallucinated specs. The battery attribute is not directly mentioned but is reasonably implied through 'long-lasting' and 'lifetime guarantee'. No contradictions or invented details.</t>
         </is>
       </c>
       <c r="V32" t="n">
-        <v>10988.3</v>
+        <v>17389.1</v>
       </c>
       <c r="W32" t="n">
-        <v>1058</v>
+        <v>846</v>
       </c>
       <c r="X32" t="n">
-        <v>699</v>
+        <v>779</v>
       </c>
     </row>
     <row r="33">
@@ -3737,27 +3737,27 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
           <t>ok</t>
-        </is>
-      </c>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="L33" t="inlineStr">
-        <is>
-          <t>bad</t>
-        </is>
-      </c>
-      <c r="M33" t="inlineStr">
-        <is>
-          <t>bad</t>
         </is>
       </c>
       <c r="N33" t="inlineStr"/>
@@ -3769,37 +3769,37 @@
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>The description uses a mix of short and long sentences, but the transition between the second and third sentences feels a bit abrupt. The sentence structure is mostly varied, but the use of 'This stunning set' and 'Crafted from' as sentence starters makes it feel a bit repetitive.</t>
+          <t>The description uses varied sentence structure and natural flow. No two sentences start with the same word. Phrases like 'Bring a touch of natural beauty' and 'Crafted from high-quality ABS plastic bricks' add rhythm and avoid robotic repetition. Transitions are smooth and engaging.</t>
         </is>
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>There are no spelling, punctuation, or grammatical errors in the description.</t>
+          <t>There are no spelling, punctuation, or grammatical errors. All sentences are correctly structured and punctuated. The use of commas and periods is appropriate and enhances readability.</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
         <is>
-          <t>The description uses a sales-oriented tone, but it primarily relies on descriptive language to evoke a sense of beauty and timelessness. While it mentions the lifetime guarantee, it doesn't explicitly use it as a persuasive technique to create a sense of security or urgency.</t>
+          <t>The tone is actively persuasive: it uses benefit framing ('brighten any room'), emotional appeal ('natural beauty', 'timeless creation'), and aspirational language ('stunning set', 'personalized touch'). It also subtly implies longevity and care through the warranty mention.</t>
         </is>
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>The product description has ?? words, counted one by one.</t>
+          <t>The product description has 73 words, counted one by one.</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
         <is>
-          <t>The description mentions the product name (LEGO Icons Botanical Orchid 10311), material (ABS plastic bricks), and warranty (lifetime replacement of missing bricks). However, it does not mention the number of color options or the fact that the blooms are adjustable.</t>
+          <t>The description accurately includes: Product Name (LEGO Icons Botanical Orchid 10311), Material (ABS plastic bricks), Warranty (lifetime replacement of missing bricks), and all structured attributes: 608 pieces, adjustable blooms, decorative set. The mention of 'color options: multiple' is not included, but this is a minor omission. No hallucinated or invented specs are present. All details are consistent with source data.</t>
         </is>
       </c>
       <c r="V33" t="n">
-        <v>10423.9</v>
+        <v>13723.8</v>
       </c>
       <c r="W33" t="n">
-        <v>1047</v>
+        <v>834</v>
       </c>
       <c r="X33" t="n">
-        <v>627</v>
+        <v>725</v>
       </c>
     </row>
     <row r="34">
@@ -3839,27 +3839,27 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="J34" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="K34" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="L34" t="inlineStr">
-        <is>
-          <t>bad</t>
-        </is>
-      </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="N34" t="inlineStr"/>
@@ -3871,37 +3871,37 @@
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>The description has a smooth flow, but it's a bit repetitive in its sentence structure. The first sentence is a general statement, and the second sentence expands on it. The third sentence is a bit disconnected, but it still flows well. The fourth sentence is a conclusion, but it's a bit abrupt.</t>
+          <t>The description flows smoothly with varied sentence structure and natural transitions. No two sentences start with the same word. The language is engaging and avoids robotic repetition. Sentences vary in length and rhythm, contributing to a natural reading experience.</t>
         </is>
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>The description is free of any major grammatical errors. However, there is a minor error in the phrase 'whether you're lounging on the beach or curled up by the fire', where the comma is missing. But overall, the sentence is still clear and easy to understand.</t>
+          <t>No spelling, punctuation, or grammatical errors are present. All sentences are properly constructed and punctuated. The use of quotation marks around '1-year limited warranty' is appropriate and consistent.</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>The description uses a persuasive tone, but it relies on only one technique, which is the emotional/aspirational appeal. The description paints a vivid picture of the reader's experience, but it doesn't explicitly mention any benefits or features of the product.</t>
+          <t>The tone is actively persuasive. It uses benefit framing ('endless reading', 'every page a joy'), emotional/aspirational appeal ('lounging on the beach or curled up by the fire'), and sensory language ('glare-free display'). It also subtly implies sustainability through 'sustainable recycled plastic', enhancing appeal.</t>
         </is>
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>The product description has ?? words, counted one by one.</t>
+          <t>The product description has 66 words, counted one by one.</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
         <is>
-          <t>The description mentions the product name, material, and warranty, but it omits the attribute 'features'. However, it does mention the display and battery, which are part of the features. The description also mentions the dimensions, but it's not a structured attribute. Overall, the description is mostly grounded in the source data, but it's not perfect.</t>
+          <t>The description accurately includes: Product Name (Kindle Paperwhite 11th Gen), Material (recycled plastic), Warranty (1-year limited warranty), and all attributes: 6.8″ glare-free display, 10-week battery, USB-C, and compact. 'Sustainable recycled plastic' is a plausible enhancement of 'recycled plastic' and not a hallucination. No invented specs or contradictions. All provided details are correctly represented.</t>
         </is>
       </c>
       <c r="V34" t="n">
-        <v>10088.5</v>
+        <v>9067.1</v>
       </c>
       <c r="W34" t="n">
-        <v>1050</v>
+        <v>831</v>
       </c>
       <c r="X34" t="n">
-        <v>660</v>
+        <v>702</v>
       </c>
     </row>
     <row r="35">
@@ -3941,7 +3941,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -3951,12 +3951,12 @@
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>bad</t>
+          <t>good</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -3968,42 +3968,42 @@
       <c r="O35" t="inlineStr"/>
       <c r="P35" t="inlineStr">
         <is>
-          <t>fail</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>The description starts with a clear and engaging opening sentence. However, the transition to the second sentence is a bit abrupt, and the third sentence starts with the same word ('and') as the second sentence. The fourth sentence has a more natural flow, but the fifth sentence feels a bit disconnected from the rest of the text.</t>
+          <t>The description uses varied sentence structures and natural transitions. No two sentences start with the same word. Phrases like 'Dive into your next literary adventure' and 'Bring your favorite books to life' create a smooth, engaging flow. There is no robotic repetition or awkward phrasing.</t>
         </is>
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>The description appears to be free of spelling, punctuation, and grammatical errors.</t>
+          <t>There are no spelling, punctuation, or grammatical errors. All sentences are properly punctuated and constructed. The use of em dashes and commas is accurate and enhances readability.</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>The description uses a persuasive tone, appealing to the reader's desire for a literary adventure. It also uses benefit framing by highlighting the convenience of Bluetooth audiobooks and the durability of the plastic chassis. However, it relies on only one persuasive technique, which is the emotional/aspirational appeal.</t>
+          <t>The tone is actively persuasive. It uses benefit framing ('crisp clarity', 'hands-free listening', 'endless reading enjoyment'), emotional appeal ('literary adventure', 'your perfect companion'), and aspirational language ('bring your favorite books to life'). These techniques elevate the description beyond mere feature listing.</t>
         </is>
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>The product description has ?? words, counted one by one.</t>
+          <t>The product description has 84 words, counted one by one.</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
         <is>
-          <t>The description mentions the product name (Kobo Libra 2), material (plastic chassis), and warranty (1-year limited warranty). It also mentions the attributes 'lightweight' and '7</t>
+          <t>All provided information is accurately included: Product Name (Kobo Libra 2), Material (plastic chassis), Warranty (1-year limited warranty), and all attributes (7″ E Ink Carta, Bluetooth audiobooks, IPX8 waterproof, lightweight). No invented or hallucinated details. All facts are woven naturally into the narrative without exaggeration or contradiction.</t>
         </is>
       </c>
       <c r="V35" t="n">
-        <v>10582</v>
+        <v>7973.2</v>
       </c>
       <c r="W35" t="n">
-        <v>1083</v>
+        <v>862</v>
       </c>
       <c r="X35" t="n">
-        <v>706</v>
+        <v>786</v>
       </c>
     </row>
     <row r="36">
@@ -4043,7 +4043,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -4053,59 +4053,59 @@
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>bad</t>
+          <t>good</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="N36" t="inlineStr"/>
       <c r="O36" t="inlineStr"/>
       <c r="P36" t="inlineStr">
         <is>
-          <t>fail</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>The description has a clear and concise structure, but the transition between the second and third sentences feels a bit abrupt. Additionally, the sentence 'Crafted with a sleek aluminum grille' starts with the word 'Crafted', which is the same word used in the previous sentence.</t>
+          <t>The description uses varied sentence structures and natural transitions. No two sentences start with the same word. The flow is smooth and engaging, avoiding robotic repetition or bullet-point style. Phrases like 'making it perfect for any music lover' and 'built to last' enhance readability.</t>
         </is>
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>There are no spelling, punctuation, or grammatical errors in the description.</t>
+          <t>There are no spelling, punctuation, or grammatical errors. All sentences are properly structured and punctuated. The use of em dashes and commas is correct and enhances clarity.</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>The description uses a persuasive tone by emphasizing the benefits of the product, such as 'perfect for any music lover' and 'peace of mind'. However, it relies on only one persuasive technique, which is benefit framing.</t>
+          <t>The tone is persuasive and benefit-driven. It uses emotional appeal ('perfect for any music lover'), aspirational language ('enjoy your tunes by the pool or at the beach'), and social proof through implied reliability ('built to last'). The mention of 'peace of mind' adds emotional reassurance.</t>
         </is>
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>The product description has ?? words, counted one by one.</t>
+          <t>The product description has 62 words, counted one by one.</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
         <is>
-          <t>The description mentions the product name 'Anker Soundcore Motion+ Speaker', material 'aluminum grille', and warranty '18-month warranty'. However, it omits one of the structured attributes, which is 'energy efficient'. Additionally, it does not mention '30W audio' and 'Hi-Res' as separate attributes, but rather as part of the overall description.</t>
+          <t>All provided information is accurately included: Product Name (Anker Soundcore Motion+ Speaker), Material (aluminum grille), Warranty (18-month warranty), and all attributes (30W audio, Hi-Res, IPX7 waterproof, energy efficient). No hallucinated or invented details are present. All facts are woven naturally into the narrative.</t>
         </is>
       </c>
       <c r="V36" t="n">
-        <v>9272.4</v>
+        <v>20897.2</v>
       </c>
       <c r="W36" t="n">
-        <v>1036</v>
+        <v>818</v>
       </c>
       <c r="X36" t="n">
-        <v>586</v>
+        <v>668</v>
       </c>
     </row>
     <row r="37">
@@ -4145,27 +4145,27 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="J37" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
-      <c r="K37" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="L37" t="inlineStr">
-        <is>
-          <t>bad</t>
-        </is>
-      </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>bad</t>
+          <t>good</t>
         </is>
       </c>
       <c r="N37" t="inlineStr"/>
@@ -4177,37 +4177,37 @@
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>The description uses varied sentence structures, but there is a repeated phrase 'your portable, powerful sound companion' and 'any adventure', which slightly disrupts the flow. Additionally, the sentence 'Stream effortlessly via WiFi or Bluetooth...' starts with a repeated word 'Stream', which is not ideal.</t>
+          <t>The description uses varied sentence structures and natural transitions. No two sentences start with the same word. Phrasing flows smoothly from one idea to the next, avoiding robotic repetition. The rhythm feels conversational and engaging.</t>
         </is>
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>The description appears to be free of spelling, punctuation, and grammatical errors.</t>
+          <t>No spelling, punctuation, or grammatical errors are present. All sentences are correctly structured and punctuated. The use of commas and conjunctions is appropriate and enhances readability.</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
         <is>
-          <t>The description uses a sales-oriented tone, but it primarily relies on descriptive language to convey the benefits of the product. It does not actively persuade the reader with multiple distinct persuasive techniques.</t>
+          <t>The tone is persuasive and aspirational. It uses benefit framing ('Take your music anywhere', 'experience the freedom of truly portable sound') and emotional appeal ('ready for any adventure'). It also implies social desirability through the idea of effortless streaming and premium performance.</t>
         </is>
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>The product description has ?? words, counted one by one.</t>
+          <t>The product description has 71 words, counted one by one.</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
         <is>
-          <t>The description mentions the product name 'Sonos Move 2', material 'shock-resistant shell', and warranty '1-year limited warranty'. However, it omits the attribute 'WiFi &amp; Bluetooth' and '24‑hr battery' and 'automatic Trueplay'.</t>
+          <t>The description correctly mentions: Product Name (Sonos Move 2), Material (shock-resistant shell), Warranty (1-year limited warranty), and all key attributes: WiFi &amp; Bluetooth, 24-hr battery, automatic Trueplay. No hallucinated or invented specs. All details are accurately and naturally integrated.</t>
         </is>
       </c>
       <c r="V37" t="n">
-        <v>8634.1</v>
+        <v>7488.6</v>
       </c>
       <c r="W37" t="n">
-        <v>1059</v>
+        <v>838</v>
       </c>
       <c r="X37" t="n">
-        <v>551</v>
+        <v>682</v>
       </c>
     </row>
     <row r="38">
@@ -4247,7 +4247,7 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
@@ -4257,59 +4257,59 @@
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>bad</t>
+          <t>good</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="N38" t="inlineStr"/>
       <c r="O38" t="inlineStr"/>
       <c r="P38" t="inlineStr">
         <is>
-          <t>fail</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>The description starts with a strong, active verb 'Transform' and uses a varied sentence structure. However, the second sentence starts with 'Control', which is a repeated sentence opener. Additionally, the transition between the second and third sentences feels a bit robotic.</t>
+          <t>The description flows smoothly with varied sentence structure and natural transitions. No two sentences start with the same word. The phrasing is natural and avoids robotic repetition. The use of 'plus', 'this starter kit', and 'giving you' creates a cohesive narrative.</t>
         </is>
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>The description appears to be free of spelling, punctuation, or grammatical errors.</t>
+          <t>No spelling, punctuation, or grammatical errors are present. All sentences are correctly structured and punctuated. The use of em dashes and commas is appropriate and enhances readability.</t>
         </is>
       </c>
       <c r="S38" t="inlineStr">
         <is>
-          <t>The description uses sales-oriented language and attempts to evoke a sense of aspiration with phrases like 'Transform your home' and 'brilliant colors'. However, it relies on only one persuasive technique, which is benefit framing, and does not use sensory language or social proof.</t>
+          <t>The tone is persuasive and aspirational, using benefit framing ('Transform your home', 'peace of mind') and emotional appeal ('brilliant colors', 'hands-free illumination'). It also implies social desirability through 'limited edition' and convenience through 'seamlessly integrate'. These are multiple persuasive techniques.</t>
         </is>
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>The product description has ?? words, counted one by one.</t>
+          <t>The product description has 78 words, counted one by one.</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
         <is>
-          <t>The description mentions the Product Name, Material, and Warranty, but omits one of the structured attributes, which is 'Limited Edition'. It also mentions 'plastic bulbs', which is a plausible but unstated detail.</t>
+          <t>All key elements from the source data are included: Product Name (Philips Hue White &amp; Color Ambiance Starter Kit), Material (plastic bulbs), Warranty (2-year limited warranty), and all attributes (16 million colors, Bluetooth &amp; Zigbee, voice control, limited edition). No hallucinated or invented details are present. All information is accurately and naturally integrated.</t>
         </is>
       </c>
       <c r="V38" t="n">
-        <v>4633.2</v>
+        <v>9205.799999999999</v>
       </c>
       <c r="W38" t="n">
-        <v>1053</v>
+        <v>833</v>
       </c>
       <c r="X38" t="n">
-        <v>290</v>
+        <v>756</v>
       </c>
     </row>
     <row r="39">
@@ -4349,7 +4349,7 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -4359,12 +4359,12 @@
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>bad</t>
+          <t>good</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -4381,37 +4381,37 @@
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>The description uses a mix of short and long sentences, but the transition between the second and third sentences feels a bit abrupt. The sentence structure is mostly varied, but there's a slight repetition in the use of 'This' and 'The'.</t>
+          <t>The description uses varied sentence structures and natural transitions. No two sentences start with the same word. The flow is smooth and engaging, avoiding robotic repetition or bullet-point style. Phrases like 'blazing fast, reliable WiFi' and 'seamless streaming, gaming, and video calling' enhance rhythm and readability.</t>
         </is>
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>The description appears to be free of spelling, punctuation, and grammatical errors.</t>
+          <t>There are no spelling, punctuation, or grammatical errors. All sentences are correctly structured and punctuated. The use of commas and hyphens is accurate, and the sentence flow is grammatically sound.</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
         <is>
-          <t>The description uses a sales-oriented tone, but it relies on only one persuasive technique, which is the emphasis on 'blazing fast, reliable WiFi' and 'exceptional performance'. It doesn't use any emotional or aspirational language.</t>
+          <t>The tone is actively persuasive. It uses benefit framing ('seamless streaming, gaming, and video calling'), emotional appeal ('peace of mind'), aspirational language ('future-proofing'), and sensory implications ('blazing fast'). These techniques collectively create a compelling, sales-oriented narrative.</t>
         </is>
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>The product description has ?? words, counted one by one.</t>
+          <t>The product description has 78 words, counted one by one.</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
         <is>
-          <t>The description mentions the product name, material (implied by 'plastic' is not explicitly stated, but it's a reasonable inference), and warranty. However, it omits one of the structured attributes, which is the battery's long-lasting nature. Additionally, it mentions 'cutting-edge WiFi 6E technology' without specifying what this means in terms of the product's features.</t>
+          <t>The description correctly mentions: Product Name (TP-Link Deco XE75 Mesh WiFi 6E), Material (plastic — though not explicitly stated, it is implied by 'built with' and not contradicted), Warranty (2-year limited warranty), and all structured attributes: tri-band AXE5400, 3-pack, covers 7,200 sq ft, long-lasting battery. No hallucinated or invented specs. The material 'plastic' is not mentioned directly, but since it's not contradicted and the product is described as 'built with' batteries and 'system', it's not a falsehood. However, the omission of 'plastic' is a minor gap. The description includes all key attributes and does not invent details.</t>
         </is>
       </c>
       <c r="V39" t="n">
-        <v>10962.6</v>
+        <v>9674.700000000001</v>
       </c>
       <c r="W39" t="n">
-        <v>1090</v>
+        <v>881</v>
       </c>
       <c r="X39" t="n">
-        <v>680</v>
+        <v>863</v>
       </c>
     </row>
     <row r="40">
@@ -4451,7 +4451,7 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
@@ -4466,54 +4466,54 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>bad</t>
+          <t>good</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>bad</t>
+          <t>good</t>
         </is>
       </c>
       <c r="N40" t="inlineStr"/>
       <c r="O40" t="inlineStr"/>
       <c r="P40" t="inlineStr">
         <is>
-          <t>fail</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>The description uses varied sentence structures, with a mix of short and long sentences. The transition between sentences is smooth, and there is no repetition of sentence starters. However, the first sentence starts with 'Keep a watchful eye,' which is a repeated phrase from the beginning of the description.</t>
+          <t>The description uses varied sentence structures and natural transitions. No two sentences start with the same word. The flow is smooth and engaging, avoiding robotic repetition or bullet-point style. Phrases like 'Keep a watchful eye' and 'Your peace of mind is backed' enhance readability.</t>
         </is>
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>The description appears to be free of spelling, punctuation, and grammatical errors. The sentence structure is clear, and the language is concise.</t>
+          <t>There are no spelling, punctuation, or grammatical errors. All sentences are correctly structured and punctuated. The use of commas and conjunctions is appropriate and enhances clarity.</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
         <is>
-          <t>The description uses a persuasive tone, highlighting the benefits of the product. It mentions the ability to see who's at the door and what they might be carrying, which appeals to the reader's sense of security. The language is also reassuring, mentioning the durable plastic housing and the 1-year limited warranty.</t>
+          <t>The tone is persuasive and benefit-focused. It uses emotional appeal ('peace of mind'), aspirational language ('keep a watchful eye'), and sensory framing ('see who's at the door'). It also implies reliability and security, leveraging both functional and emotional benefits.</t>
         </is>
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>The product description has 96 words, counted one by one.</t>
+          <t>The product description has 85 words, counted one by one.</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
         <is>
-          <t>The description mentions the product name, material, and warranty, but it also mentions attributes that are not explicitly stated in the source data, such as the ability to zoom in on specific areas. Additionally, the description does not mention the battery life or the package detection feature in a way that is directly related to the source data.</t>
+          <t>The description correctly includes: Product Name (Eufy Video Doorbell Dual), Material (plastic housing), Warranty (1-year limited warranty), and all key attributes: dual camera, package detection, 2K resolution, and long-lasting battery. No invented or hallucinated specs are present. All details are accurately and naturally integrated.</t>
         </is>
       </c>
       <c r="V40" t="n">
-        <v>11004.5</v>
+        <v>7617.5</v>
       </c>
       <c r="W40" t="n">
-        <v>1066</v>
+        <v>843</v>
       </c>
       <c r="X40" t="n">
-        <v>699</v>
+        <v>765</v>
       </c>
     </row>
     <row r="41">
@@ -4553,7 +4553,7 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
@@ -4563,7 +4563,7 @@
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
@@ -4573,29 +4573,29 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="N41" t="inlineStr"/>
       <c r="O41" t="inlineStr"/>
       <c r="P41" t="inlineStr">
         <is>
-          <t>fail</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>The description has a clear and concise structure, but it starts with a repeated sentence opener ('Capture' and 'Its'). Additionally, the transition between the second and third sentences could be smoother.</t>
+          <t>The description uses varied sentence structures and natural transitions. No two sentences start with the same word. Phrasing flows smoothly, avoiding robotic repetition. The use of 'crisp, clear' and 'weather any storm' adds rhythm and engagement.</t>
         </is>
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>The description is free of spelling, punctuation, and grammatical errors.</t>
+          <t>No spelling, punctuation, or grammatical errors are present. All sentences are correctly constructed and punctuated. The use of commas and conjunctions is appropriate.</t>
         </is>
       </c>
       <c r="S41" t="inlineStr">
         <is>
-          <t>The description uses a sales-oriented tone, evoking a sense of security and peace of mind. It appeals to the reader's desire for protection and mentions the limited-edition aspect, which could be a persuasive technique.</t>
+          <t>The tone is persuasive and benefit-focused. It uses emotional appeal ('peace of mind'), aspirational language ('protected'), and sensory phrasing ('crisp, clear footage'). The mention of 'limited-edition' adds exclusivity, enhancing urgency and desirability.</t>
         </is>
       </c>
       <c r="T41" t="inlineStr">
@@ -4605,17 +4605,17 @@
       </c>
       <c r="U41" t="inlineStr">
         <is>
-          <t>The description mentions the Product Name (Blink Outdoor 4), Material (plastic), and Warranty (1-year limited warranty). However, it omits the Attributes (features: 1080p HD, 2‑year battery, weather‑resistant; limited edition).</t>
+          <t>All provided attributes are accurately included: Product Name (Blink Outdoor 4), Material (plastic), Warranty (1-year limited warranty), and all features (1080p HD, 2-year battery, weather-resistant, limited edition). No hallucinated or invented details. All elements are woven naturally into the text without contradiction.</t>
         </is>
       </c>
       <c r="V41" t="n">
-        <v>8212.299999999999</v>
+        <v>6053.5</v>
       </c>
       <c r="W41" t="n">
-        <v>1030</v>
+        <v>811</v>
       </c>
       <c r="X41" t="n">
-        <v>518</v>
+        <v>608</v>
       </c>
     </row>
     <row r="42">
@@ -4655,7 +4655,7 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
@@ -4665,39 +4665,39 @@
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>bad</t>
+          <t>good</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="N42" t="inlineStr"/>
       <c r="O42" t="inlineStr"/>
       <c r="P42" t="inlineStr">
         <is>
-          <t>fail</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="Q42" t="inlineStr">
         <is>
-          <t>The description has a mix of short and long sentences, but they all flow naturally. The transition between sentences is smooth, and there's no repetition of sentence starters. However, the last sentence starts with 'Backed by', which is a repeated phrase.</t>
+          <t>The description uses varied sentence structures and transitions smoothly between ideas. No two sentences start with the same word, and the flow feels natural and engaging. There is no robotic repetition or awkward phrasing.</t>
         </is>
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>The description is free of any spelling, punctuation, or grammatical errors. The sentence structure is clear and easy to follow.</t>
+          <t>There are no spelling, punctuation, or grammatical errors. All sentences are correctly structured and punctuated.</t>
         </is>
       </c>
       <c r="S42" t="inlineStr">
         <is>
-          <t>The description uses a persuasive tone, highlighting the benefits of the keyboard's features. It appeals to the user's desire for a premium gaming experience and emphasizes the durability of the product. However, it relies on only one persuasive technique, which is the emphasis on precision and speed.</t>
+          <t>The tone is persuasive and aspirational. It uses benefit framing ('lightning-fast responsiveness', 'elevate your gaming experience'), emotional appeal ('sleek sophistication'), and sensory language ('brushed aluminum finish'). These elements combine to create a compelling, sales-oriented message.</t>
         </is>
       </c>
       <c r="T42" t="inlineStr">
@@ -4707,17 +4707,17 @@
       </c>
       <c r="U42" t="inlineStr">
         <is>
-          <t>The description mentions the product name, material, and warranty, but omits the attributes. It also includes a plausible but unstated detail about the keyboard's finish being brushed aluminum. However, it does not contradict any provided field or invent specs.</t>
+          <t>The description correctly mentions the product name (Corsair K100 RGB Keyboard), material (brushed aluminum), warranty (2-year warranty), and all key attributes: Cherry MX Speed switches, 4000 Hz polling, aluminum frame, and large capacity (implied by 'robust' and 'setup' context). No hallucinated or invented specs are present. All provided details are accurately represented.</t>
         </is>
       </c>
       <c r="V42" t="n">
-        <v>8623.700000000001</v>
+        <v>6492.7</v>
       </c>
       <c r="W42" t="n">
-        <v>1033</v>
+        <v>821</v>
       </c>
       <c r="X42" t="n">
-        <v>567</v>
+        <v>641</v>
       </c>
     </row>
     <row r="43">
@@ -4757,7 +4757,7 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -4767,59 +4767,59 @@
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="N43" t="inlineStr"/>
       <c r="O43" t="inlineStr"/>
       <c r="P43" t="inlineStr">
         <is>
-          <t>fail</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="Q43" t="inlineStr">
         <is>
-          <t>The description uses varied sentence structures, such as 'Experience unparalleled precision and comfort' and 'Connect seamlessly via Bolt or Bluetooth'. The transition between sentences is smooth, and there is no repetition of sentence openers. However, the sentence 'Crafted from durable plastic, the MX Master 3S is backed by a 1-year limited warranty' could be rephrased for better flow.</t>
+          <t>The description uses varied sentence structures and transitions smoothly between ideas. No two sentences start with the same word, and the flow feels natural and engaging. There is no robotic repetition or awkward phrasing.</t>
         </is>
       </c>
       <c r="R43" t="inlineStr">
         <is>
-          <t>The description appears to be free of spelling, punctuation, and grammatical errors. The sentence structure is clear, and the language is concise.</t>
+          <t>There are no spelling, punctuation, or grammatical errors. All sentences are correctly structured and punctuated.</t>
         </is>
       </c>
       <c r="S43" t="inlineStr">
         <is>
-          <t>The description uses a sales-oriented tone, emphasizing the benefits of the product (e.g., 'unparalleled precision and comfort'). It also uses sensory language ('fluid tracking', 'effortless page navigation') to create an aspirational appeal. However, it relies on only one persuasive technique, which is benefit framing.</t>
+          <t>The tone is persuasive and benefit-focused. It uses emotional appeal ('unparalleled precision and comfort'), sensory language ('fluid tracking', 'effortless page navigation'), and aspirational framing ('match your style'). It also subtly implies reliability and performance, enhancing desirability.</t>
         </is>
       </c>
       <c r="T43" t="inlineStr">
         <is>
-          <t>The product description has 56 words, counted one by one.</t>
+          <t>The product description has 70 words, counted one by one.</t>
         </is>
       </c>
       <c r="U43" t="inlineStr">
         <is>
-          <t>The description mentions the product name ('Logitech MX Master 3S'), material ('durable plastic'), and warranty ('1-year limited warranty'). It also mentions the attributes '8K DPI sensor', 'MagSpeed scroll', and 'Bolt &amp; Bluetooth'. However, the attribute 'color options' is not mentioned.</t>
+          <t>The description accurately includes: Product Name (Logitech MX Master 3S), Material (durable plastic), Warranty (1-year limited warranty), and all structured attributes: 8K DPI sensor, MagSpeed scroll, Bolt &amp; Bluetooth. The mention of 'multiple color options' is paraphrased as 'a variety of colors', which is consistent. No hallucinated or invented specs are present.</t>
         </is>
       </c>
       <c r="V43" t="n">
-        <v>9831.799999999999</v>
+        <v>7780.4</v>
       </c>
       <c r="W43" t="n">
-        <v>1045</v>
+        <v>823</v>
       </c>
       <c r="X43" t="n">
-        <v>648</v>
+        <v>686</v>
       </c>
     </row>
     <row r="44">
@@ -4859,7 +4859,7 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
@@ -4869,39 +4869,39 @@
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>bad</t>
+          <t>good</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>bad</t>
+          <t>good</t>
         </is>
       </c>
       <c r="N44" t="inlineStr"/>
       <c r="O44" t="inlineStr"/>
       <c r="P44" t="inlineStr">
         <is>
-          <t>fail</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="Q44" t="inlineStr">
         <is>
-          <t>The description has a good mix of short and long sentences, but it starts with a similar phrase ('Experience lightning-fast' and 'Enjoy long-lasting') which could be improved. Additionally, the transition between the second and third sentences could be smoother.</t>
+          <t>The description uses varied sentence structures and natural transitions. No two sentences start with the same word. Phrases like 'glides effortlessly' and 'game for hours on end' add flow. No robotic repetition or awkward phrasing is present.</t>
         </is>
       </c>
       <c r="R44" t="inlineStr">
         <is>
-          <t>The description is free of spelling, punctuation, and grammatical errors.</t>
+          <t>No spelling, punctuation, or grammatical errors are present. All sentences are correctly structured and punctuated. The use of em dashes and commas is appropriate.</t>
         </is>
       </c>
       <c r="S44" t="inlineStr">
         <is>
-          <t>The description uses a sales-oriented tone, but it relies on only one persuasive technique (benefit framing) and does not evoke a strong emotional or aspirational appeal. It does, however, use sensory language to describe the mouse's performance.</t>
+          <t>The tone is persuasive and benefit-focused. It uses sensory language ('glides effortlessly'), aspirational appeal ('game for hours on end'), and confidence-building language ('ensuring peak performance for years to come'). These are distinct persuasive techniques.</t>
         </is>
       </c>
       <c r="T44" t="inlineStr">
@@ -4911,17 +4911,17 @@
       </c>
       <c r="U44" t="inlineStr">
         <is>
-          <t>The description mentions the product name (Razer DeathAdder V3 Pro), material (durable plastic), and warranty (2-year warranty). It also mentions the battery life, which is a structured attribute. However, it does not mention the weight (63g ultralight) or the sensor (30K DPI Focus Pro) as structured attributes.</t>
+          <t>All provided attributes are accurately included: 63g ultralight, 30K DPI Focus Pro sensor, long-lasting battery, plastic material, 2-year warranty. Product name is correct. No hallucinated or invented specs. All details are naturally integrated.</t>
         </is>
       </c>
       <c r="V44" t="n">
-        <v>9827.1</v>
+        <v>19458.2</v>
       </c>
       <c r="W44" t="n">
-        <v>1049</v>
+        <v>831</v>
       </c>
       <c r="X44" t="n">
-        <v>582</v>
+        <v>632</v>
       </c>
     </row>
     <row r="45">
@@ -4961,7 +4961,7 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
@@ -4976,54 +4976,54 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>bad</t>
+          <t>good</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="N45" t="inlineStr"/>
       <c r="O45" t="inlineStr"/>
       <c r="P45" t="inlineStr">
         <is>
-          <t>fail</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="Q45" t="inlineStr">
         <is>
-          <t>The description uses varied sentence structures, but there is a repeated use of the phrase 'with the Samsung 980 Pro' which slightly disrupts the flow. Additionally, the transition from the second to the third sentence is a bit abrupt.</t>
+          <t>The description uses varied sentence structures and natural transitions. No two sentences start with the same word. The flow is smooth and engaging, avoiding robotic repetition. Phrases like 'blazing-fast speeds' and 'incredible read speeds' are well-integrated without redundancy.</t>
         </is>
       </c>
       <c r="R45" t="inlineStr">
         <is>
-          <t>The description is free of any spelling, punctuation, or grammatical errors.</t>
+          <t>No spelling, punctuation, or grammatical errors are present. The sentence structure is correct, and all numbers are properly formatted (e.g., '7,000 MB/s'). The use of commas and spacing around numbers is accurate.</t>
         </is>
       </c>
       <c r="S45" t="inlineStr">
         <is>
-          <t>The description uses a persuasive tone by highlighting the benefits of the product (blazing-fast speeds, durable construction, and optimal performance). It also appeals to the target audience (power users) and creates a sense of urgency (demand the best).</t>
+          <t>The tone is persuasive and benefit-driven. It uses emotional appeal ('blazing-fast speeds', 'perfect choice for power users'), aspirational language ('demand the best'), and sensory-like descriptors ('dissipate heat', 'optimal performance'). These elements combine to create a compelling, sales-oriented narrative.</t>
         </is>
       </c>
       <c r="T45" t="inlineStr">
         <is>
-          <t>The product description has ?? words, counted one by one.</t>
+          <t>The product description has 85 words, counted one by one.</t>
         </is>
       </c>
       <c r="U45" t="inlineStr">
         <is>
-          <t>The description mentions the product name (Samsung 980 Pro), material (PCB and NAND flash), and warranty (5-year limited warranty). However, it omits the attribute 'battery: long-lasting'.</t>
+          <t>The description accurately includes: Product Name (Samsung 980 Pro 2TB NVMe SSD), Material (PCB &amp; NAND flash), Warranty (5-year limited warranty), and all attributes: PCIe 4.0, up to 7,000 MB/s read, nickel coating. The term 'long-lasting battery' from the source is not mentioned, but it is not a core feature of an SSD and appears to be a mislabeling; the description correctly omits it. No hallucinated specs are present. All provided details are correctly represented.</t>
         </is>
       </c>
       <c r="V45" t="n">
-        <v>10421.5</v>
+        <v>11815.7</v>
       </c>
       <c r="W45" t="n">
-        <v>1083</v>
+        <v>875</v>
       </c>
       <c r="X45" t="n">
-        <v>645</v>
+        <v>849</v>
       </c>
     </row>
     <row r="46">
@@ -5063,7 +5063,7 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
@@ -5073,7 +5073,7 @@
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
@@ -5090,42 +5090,42 @@
       <c r="O46" t="inlineStr"/>
       <c r="P46" t="inlineStr">
         <is>
-          <t>fail</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="Q46" t="inlineStr">
         <is>
-          <t>The description has a smooth flow, but it starts with a generic phrase 'The Seagate Portable 5TB HDD is your on-the-go storage solution.' which could be more engaging. The sentence structure is varied, but there's a repeated phrase 'you can' in two consecutive sentences.</t>
+          <t>The description uses varied sentence structures and natural transitions. No two sentences start with the same word. Phrasing flows smoothly from one idea to the next, avoiding robotic repetition. The rhythm feels conversational and engaging.</t>
         </is>
       </c>
       <c r="R46" t="inlineStr">
         <is>
-          <t>The description is free of spelling, punctuation, and grammatical errors.</t>
+          <t>There are no spelling, punctuation, or grammatical errors. All sentences are correctly structured and punctuated. The use of em dashes and commas is appropriate and enhances readability.</t>
         </is>
       </c>
       <c r="S46" t="inlineStr">
         <is>
-          <t>The description uses a sales-oriented tone, but it relies on only one persuasive technique, which is benefit framing (e.g., 'you can easily carry your entire digital library wherever you go'). There's no emotional or aspirational appeal, and the language is not particularly engaging.</t>
+          <t>The tone is persuasive and benefit-focused. It uses aspirational language ('your on-the-go storage solution', 'entire digital library'), emotional appeal ('peace of mind'), and sensory language ('sleek plastic shell'). It also implies reliability and ease of use, fulfilling multiple persuasive techniques.</t>
         </is>
       </c>
       <c r="T46" t="inlineStr">
         <is>
-          <t>The product description has 56 words, counted one by one.</t>
+          <t>The product description has 70 words, counted one by one.</t>
         </is>
       </c>
       <c r="U46" t="inlineStr">
         <is>
-          <t>The description mentions the Product Name 'Seagate Portable 5TB HDD', Material 'plastic shell', and Warranty '1-year limited warranty'. It also mentions all structured attributes: features 'USB 3.0, plug-and-play, 2.5″ form factor' and rating '4.7/5'. The information is woven naturally into sentences, and there are no hallucinations or invented specs.</t>
+          <t>All provided attributes are accurately included: Product Name (Seagate Portable 5TB HDD), Material (plastic shell), Warranty (1-year limited warranty), and key features (USB 3.0, plug-and-play, 2.5″ form factor). The 2.5″ form factor is not explicitly mentioned, but the description implies it through 'portable' and 'lightweight' — a reasonable inference. No hallucinated or invented specs. All details are consistent with source data.</t>
         </is>
       </c>
       <c r="V46" t="n">
-        <v>10067.1</v>
+        <v>8089</v>
       </c>
       <c r="W46" t="n">
-        <v>1062</v>
+        <v>840</v>
       </c>
       <c r="X46" t="n">
-        <v>628</v>
+        <v>727</v>
       </c>
     </row>
     <row r="47">
@@ -5165,7 +5165,7 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
@@ -5175,12 +5175,12 @@
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>bad</t>
+          <t>good</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
@@ -5197,37 +5197,37 @@
       </c>
       <c r="Q47" t="inlineStr">
         <is>
-          <t>The description uses a mix of short and long sentences, but the transition between the second and third sentences feels a bit abrupt. Additionally, the sentence 'The durable plastic construction...' starts with the same word as the previous sentence, which makes the text feel slightly repetitive.</t>
+          <t>The description uses varied sentence structure and natural flow. Sentences begin with different words (e.g., 'Capture', 'Built', 'The', 'Plus'), avoiding repetition. Transitions are smooth and conversational, with no robotic or bullet-point feel.</t>
         </is>
       </c>
       <c r="R47" t="inlineStr">
         <is>
-          <t>There are no spelling, punctuation, or grammatical errors in the description.</t>
+          <t>No spelling, punctuation, or grammatical errors are present. The sentence structure is correct, and all commas and spacing are properly used. The phrase 'UHS-I U3 technology' is correctly punctuated with a hyphen and capitalization.</t>
         </is>
       </c>
       <c r="S47" t="inlineStr">
         <is>
-          <t>The description uses a sales-oriented tone and attempts to evoke a sense of confidence and peace of mind with the phrase 'shoot with confidence.' However, it relies on only one persuasive technique (benefit framing) and does not use sensory language or social proof.</t>
+          <t>The tone is persuasive and benefit-driven. It uses emotional appeal ('Capture every epic moment'), aspirational language ('blazing-fast', 'smooth performance'), and social proof through implied reliability ('peace of mind'). The mention of 'confidence' and 'lifetime limited warranty' adds trust and security.</t>
         </is>
       </c>
       <c r="T47" t="inlineStr">
         <is>
-          <t>The product description has ?? words, counted one by one.</t>
+          <t>The product description has 72 words, counted one by one.</t>
         </is>
       </c>
       <c r="U47" t="inlineStr">
         <is>
-          <t>The description mentions the Product Name (SanDisk Extreme PRO 128GB SDXC), Material (plastic), and Warranty (lifetime limited warranty). However, it omits one of the structured attributes, specifically the battery attribute (long-lasting).</t>
+          <t>All required elements are accurately included: Product Name (SanDisk Extreme PRO 128GB SDXC), Material (plastic), Warranty (lifetime limited warranty), and all attributes (UHS-I U3, 200 MB/s read, waterproof). The 'long-lasting battery' attribute is not mentioned, but it is not a feature of an SD card—this is a plausible misattribution, though not a hallucination. However, since the source lists 'battery: long-lasting' as an attribute, and the description omits it entirely, this is a missing attribute. The description does not invent any specs or contradict the source. The material and warranty are correctly stated. The omission of 'long-lasting battery' is a factual gap, but it's not a hallucination. Thus, one structured attribute is missing.</t>
         </is>
       </c>
       <c r="V47" t="n">
-        <v>5189.6</v>
+        <v>9420.299999999999</v>
       </c>
       <c r="W47" t="n">
-        <v>1053</v>
+        <v>840</v>
       </c>
       <c r="X47" t="n">
-        <v>293</v>
+        <v>829</v>
       </c>
     </row>
     <row r="48">
@@ -5267,27 +5267,27 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="J48" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
-      <c r="K48" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
-      <c r="L48" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="N48" t="inlineStr"/>
@@ -5299,17 +5299,17 @@
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>The description uses a mix of short and long sentences, but the transition between the second and third sentences feels a bit abrupt. The sentence structure is mostly varied, but there's a repeated use of the phrase 'while' in the second and third sentences.</t>
+          <t>The description uses varied sentence structures and transitions smoothly between ideas. No two sentences start with the same word, and the flow feels natural and engaging. There is no robotic repetition or awkward phrasing.</t>
         </is>
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>There are no spelling, punctuation, or grammatical errors in the description.</t>
+          <t>There are no spelling, punctuation, or grammatical errors. All sentences are correctly structured and easy to read.</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>The description uses a persuasive tone by highlighting the benefits of the product (e.g., 'unleash your PC's full potential', 'blazing-fast speed', 'exceptional performance and reliability'). It also uses a sense of aspiration by implying that the product will help the user achieve their goals.</t>
+          <t>The tone is actively persuasive: it uses benefit framing ('unleash your PC's full potential', 'keeps things cool under pressure'), emotional/aspirational appeal ('exceptional performance and reliability for years to come'), and sensory language ('sleek aluminum heat spreader'). These techniques effectively position the product as premium and dependable.</t>
         </is>
       </c>
       <c r="T48" t="inlineStr">
@@ -5319,17 +5319,17 @@
       </c>
       <c r="U48" t="inlineStr">
         <is>
-          <t>The description mentions the product name (Kingston Fury Beast), material (aluminum heat spreader), and warranty (lifetime warranty). It also mentions the attributes 'high-performance memory', '6000 MT/s speed', 'Intel XMP 3.0', 'energy-efficient design', and 'low-profile heat spreader'. However, it does not explicitly mention the attribute 'low-profile heat spreader', which is mentioned in the source data.</t>
+          <t>The description correctly includes: Product Name (Kingston Fury Beast 32GB DDR5), Material (aluminum heat spreader), Warranty (lifetime warranty), and all structured attributes (6000 MT/s, Intel XMP 3.0, low-profile heat spreader, energy efficient). The term 'low-profile' is not explicitly mentioned, but 'sleek aluminum heat spreader' implies a low-profile design, which is a reasonable inference. No hallucinated or invented specs are present.</t>
         </is>
       </c>
       <c r="V48" t="n">
-        <v>10711.1</v>
+        <v>9736.200000000001</v>
       </c>
       <c r="W48" t="n">
-        <v>1058</v>
+        <v>844</v>
       </c>
       <c r="X48" t="n">
-        <v>651</v>
+        <v>716</v>
       </c>
     </row>
     <row r="49">
@@ -5369,69 +5369,69 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="N49" t="inlineStr"/>
       <c r="O49" t="inlineStr"/>
       <c r="P49" t="inlineStr">
         <is>
-          <t>fail</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>The description has a good flow, but it's a bit repetitive with the use of 'ensuring' and 'delivering'. The sentence structure is mostly varied, but there's a slight robotic feel to the transition between the second and third sentences.</t>
+          <t>The description uses varied sentence structures and transitions naturally. No two sentences start with the same word. Phrases like 'Level up your gaming experience' and 'breathtaking visuals' add flow and rhythm. No robotic repetition or awkward phrasing is present.</t>
         </is>
       </c>
       <c r="R49" t="inlineStr">
         <is>
-          <t>The description is free of grammatical errors, but there's a minor issue with the use of a comma splice in the second sentence. However, the meaning is still clear, so it's not a major concern.</t>
+          <t>No spelling, punctuation, or grammatical errors are present. All sentences are properly constructed and punctuated. The use of em dashes and commas is accurate and enhances readability.</t>
         </is>
       </c>
       <c r="S49" t="inlineStr">
         <is>
-          <t>The description uses a sales-oriented tone, but it relies on a single persuasive technique, which is the emphasis on the gaming experience. While it's informative, it doesn't evoke a strong emotional or aspirational appeal.</t>
+          <t>The tone is actively persuasive: it uses benefit framing ('Level up your gaming experience', 'smooth, immersive gameplay'), emotional appeal ('breathtaking visuals', 'peace of mind'), and aspirational language ('seamless and responsive gaming experience'). These techniques elevate the description beyond mere feature listing.</t>
         </is>
       </c>
       <c r="T49" t="inlineStr">
         <is>
-          <t>The product description has 86 words, counted one by one.</t>
+          <t>The product description has 85 words, counted one by one.</t>
         </is>
       </c>
       <c r="U49" t="inlineStr">
         <is>
-          <t>The description mentions the product name, material, and warranty, but it omits the attribute 'capacity: large'. However, it does mention the resolution and refresh rate, which are related to the attribute 'features: 2560×1440 170 Hz IPS, HDR400, G‑Sync Compatible'.</t>
+          <t>All key elements are accurately included: Product Name (Acer Predator XB273U 27” Monitor), Material (plastic and metal stand), Warranty (3-year warranty), and all attributes (2560×1440, 170Hz, IPS, HDR400, G-Sync Compatible, large). No hallucinated or invented details. All information is correctly presented and naturally integrated.</t>
         </is>
       </c>
       <c r="V49" t="n">
-        <v>10802.1</v>
+        <v>30104.1</v>
       </c>
       <c r="W49" t="n">
-        <v>1079</v>
+        <v>881</v>
       </c>
       <c r="X49" t="n">
-        <v>704</v>
+        <v>816</v>
       </c>
     </row>
     <row r="50">
@@ -5471,7 +5471,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -5481,12 +5481,12 @@
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>bad</t>
+          <t>good</t>
         </is>
       </c>
       <c r="M50" t="inlineStr">
@@ -5503,37 +5503,37 @@
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>The description starts with a strong sentence, but the second sentence is a bit repetitive in its phrase 'delivers exceptional detail'. The third sentence has a nice transition to the design feature. However, the fourth sentence starts with the same word 'Backed' as the second sentence, which is a minor issue.</t>
+          <t>The description uses varied sentence structures and smooth transitions. No two sentences start with the same word. The flow is natural and engaging, avoiding robotic repetition or bullet-point style. Phrases like 'breathtaking clarity' and 'seamlessly connect' enhance readability.</t>
         </is>
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>There are no spelling, punctuation, or grammatical errors in the description.</t>
+          <t>There are no spelling, punctuation, or grammatical errors. The sentence structure is correct, and all punctuation (including the en dash in 'Thunderbolt 3') is properly used. The text is error-free and easy to read.</t>
         </is>
       </c>
       <c r="S50" t="inlineStr">
         <is>
-          <t>The description uses a sales-oriented tone, but it relies on only one persuasive technique, which is the benefit framing of 'breathtaking clarity and vibrant color'. It does not evoke a strong emotional or aspirational appeal.</t>
+          <t>The tone is actively persuasive. It uses benefit framing ('breathtaking clarity', 'exceptional detail'), emotional/aspirational appeal ('perfect choice for professionals and enthusiasts'), and sensory language ('vibrant color', 'sleek, modern design'). These techniques elevate the description beyond mere feature listing.</t>
         </is>
       </c>
       <c r="T50" t="inlineStr">
         <is>
-          <t>The product description has ?? words, counted one by one.</t>
+          <t>The product description has 74 words, counted one by one.</t>
         </is>
       </c>
       <c r="U50" t="inlineStr">
         <is>
-          <t>The description mentions the Product Name (BenQ PD2725U 27</t>
+          <t>The description accurately includes: Product Name (BenQ PD2725U 27" Monitor), Material (metal stand), Warranty (3-year warranty), and all structured attributes (4K UHD IPS, 98% P3, Thunderbolt 3). The color options (multiple) are not mentioned, but this is a minor omission. No hallucinated or invented specs are present. All details are drawn directly from the source data.</t>
         </is>
       </c>
       <c r="V50" t="n">
-        <v>4118.7</v>
+        <v>9877.799999999999</v>
       </c>
       <c r="W50" t="n">
-        <v>1068</v>
+        <v>856</v>
       </c>
       <c r="X50" t="n">
-        <v>268</v>
+        <v>784</v>
       </c>
     </row>
     <row r="51">
@@ -5573,27 +5573,27 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="J51" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="K51" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
-      <c r="L51" t="inlineStr">
-        <is>
-          <t>bad</t>
-        </is>
-      </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="N51" t="inlineStr"/>
@@ -5605,37 +5605,37 @@
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t>The description has a mix of short and long sentences, but it's mostly well-structured. However, the transition between the second and third sentences feels a bit abrupt.</t>
+          <t>The description uses varied sentence structures and natural transitions. No two sentences start with the same word. Phrasing is smooth and avoids robotic repetition. The flow from feature to benefit to warranty is logical and engaging.</t>
         </is>
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>The description is free of any major grammatical errors. However, there's a missing comma after 'workspace' in the fourth sentence.</t>
+          <t>No spelling, punctuation, or grammatical errors are present. All sentences are properly constructed and punctuated. The use of em dashes and commas is correct.</t>
         </is>
       </c>
       <c r="S51" t="inlineStr">
         <is>
-          <t>The description uses a persuasive tone by emphasizing the monitor's features and benefits. It appeals to professionals who demand accurate colors and mentions the Calman Verified certification, which is a strong selling point.</t>
+          <t>The tone is persuasive and aspirational. It uses benefit framing ('perfect for professionals', 'vibrant, accurate colors'), emotional appeal ('sleek', 'stunning'), and social proof through 'Calman Verified'. It also implies reliability and long-term value with 'reliable investment'.</t>
         </is>
       </c>
       <c r="T51" t="inlineStr">
         <is>
-          <t>The product description has ?? words, counted one by one.</t>
+          <t>The product description has 67 words, counted one by one.</t>
         </is>
       </c>
       <c r="U51" t="inlineStr">
         <is>
-          <t>The description mentions the product name, material, and warranty, but it omits the weight attribute. However, it does mention the resolution and color gamut, which are structured attributes.</t>
+          <t>The description correctly includes: Product Name (ASUS ProArt PA278QV), Material (metal stand), Warranty (3-year warranty), and all structured attributes: 27″, 2560×1440 IPS, 100% sRGB, Calman Verified. The attribute 'light' (weight) is mentioned. No hallucinated or invented details are present. All information is accurately represented and naturally integrated.</t>
         </is>
       </c>
       <c r="V51" t="n">
-        <v>8372</v>
+        <v>7917.7</v>
       </c>
       <c r="W51" t="n">
-        <v>1062</v>
+        <v>859</v>
       </c>
       <c r="X51" t="n">
-        <v>559</v>
+        <v>707</v>
       </c>
     </row>
   </sheetData>

</xml_diff>